<commit_message>
Improve drag and drop and image fitting, pricing
</commit_message>
<xml_diff>
--- a/data/copypro_kodai.xlsx
+++ b/data/copypro_kodai.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\deima\Downloads\copypro_tools_complete_final_bundle\data\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\deima\Downloads\copypro_tools_final_github_bundle\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="11_3B4A8E2EF7B1EBE3EABC0ACE97115682C7D972DC" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{62E82CA7-65C5-4A0D-B296-E24DAC4FE08E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="3855" yWindow="3855" windowWidth="21600" windowHeight="11385" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Items" sheetId="1" r:id="rId1"/>
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1655" uniqueCount="838">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1655" uniqueCount="839">
   <si>
     <t>category</t>
   </si>
@@ -935,9 +935,6 @@
     <t>Karštas laminatas</t>
   </si>
   <si>
-    <t>Karstas laminatas</t>
-  </si>
-  <si>
     <t>4917</t>
   </si>
   <si>
@@ -968,9 +965,6 @@
     <t>160 gsm spalvotas A4 popierius</t>
   </si>
   <si>
-    <t>966</t>
-  </si>
-  <si>
     <t>SRA3 lipdukas</t>
   </si>
   <si>
@@ -2535,13 +2529,22 @@
   </si>
   <si>
     <t>Nekeiskite stulpelių pavadinimų. Naujas eilutes pridėkite lentelės apačioje.</t>
+  </si>
+  <si>
+    <t>180gsm</t>
+  </si>
+  <si>
+    <t>Satinas ir blizgus fotopopierius</t>
+  </si>
+  <si>
+    <t>Karstas laminatas 2x</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2">
+  <fonts count="3">
     <font>
       <sz val="11"/>
       <name val="Carlito"/>
@@ -2550,6 +2553,10 @@
       <b/>
       <sz val="11"/>
       <color rgb="FFFFFFFF"/>
+      <name val="Carlito"/>
+    </font>
+    <font>
+      <sz val="8"/>
       <name val="Carlito"/>
     </font>
   </fonts>
@@ -5489,20 +5496,20 @@
         <v>249</v>
       </c>
       <c r="B127" s="1" t="s">
-        <v>270</v>
+        <v>294</v>
       </c>
       <c r="C127" s="4" t="s">
-        <v>271</v>
+        <v>295</v>
       </c>
       <c r="D127" s="5">
-        <v>2.4</v>
+        <v>2.35</v>
       </c>
       <c r="E127" s="1"/>
       <c r="F127" s="1" t="s">
         <v>261</v>
       </c>
       <c r="G127" s="1" t="s">
-        <v>258</v>
+        <v>296</v>
       </c>
       <c r="H127" s="1" t="s">
         <v>12</v>
@@ -5514,20 +5521,20 @@
         <v>249</v>
       </c>
       <c r="B128" s="1" t="s">
-        <v>272</v>
+        <v>297</v>
       </c>
       <c r="C128" s="4" t="s">
-        <v>273</v>
+        <v>298</v>
       </c>
       <c r="D128" s="5">
-        <v>2.5499999999999998</v>
+        <v>2.2999999999999998</v>
       </c>
       <c r="E128" s="1"/>
       <c r="F128" s="1" t="s">
         <v>264</v>
       </c>
       <c r="G128" s="1" t="s">
-        <v>258</v>
+        <v>296</v>
       </c>
       <c r="H128" s="1" t="s">
         <v>12</v>
@@ -5539,45 +5546,45 @@
         <v>249</v>
       </c>
       <c r="B129" s="1" t="s">
-        <v>274</v>
+        <v>270</v>
       </c>
       <c r="C129" s="4" t="s">
-        <v>275</v>
+        <v>271</v>
       </c>
       <c r="D129" s="5">
-        <v>3.2</v>
+        <v>2.4</v>
       </c>
       <c r="E129" s="1"/>
       <c r="F129" s="1" t="s">
-        <v>264</v>
+        <v>261</v>
       </c>
       <c r="G129" s="1" t="s">
-        <v>275</v>
+        <v>836</v>
       </c>
       <c r="H129" s="1" t="s">
         <v>12</v>
       </c>
       <c r="I129" s="1"/>
     </row>
-    <row r="130" spans="1:9" ht="28.5">
+    <row r="130" spans="1:9">
       <c r="A130" s="1" t="s">
         <v>249</v>
       </c>
       <c r="B130" s="1" t="s">
-        <v>276</v>
+        <v>272</v>
       </c>
       <c r="C130" s="4" t="s">
-        <v>277</v>
+        <v>273</v>
       </c>
       <c r="D130" s="5">
-        <v>2.8</v>
+        <v>2.5499999999999998</v>
       </c>
       <c r="E130" s="1"/>
       <c r="F130" s="1" t="s">
-        <v>261</v>
+        <v>264</v>
       </c>
       <c r="G130" s="1" t="s">
-        <v>277</v>
+        <v>836</v>
       </c>
       <c r="H130" s="1" t="s">
         <v>12</v>
@@ -5589,19 +5596,21 @@
         <v>249</v>
       </c>
       <c r="B131" s="1" t="s">
-        <v>278</v>
+        <v>274</v>
       </c>
       <c r="C131" s="4" t="s">
-        <v>279</v>
+        <v>275</v>
       </c>
       <c r="D131" s="5">
-        <v>3.3</v>
+        <v>3.2</v>
       </c>
       <c r="E131" s="1"/>
       <c r="F131" s="1" t="s">
-        <v>252</v>
-      </c>
-      <c r="G131" s="1"/>
+        <v>264</v>
+      </c>
+      <c r="G131" s="1" t="s">
+        <v>837</v>
+      </c>
       <c r="H131" s="1" t="s">
         <v>12</v>
       </c>
@@ -5612,20 +5621,20 @@
         <v>249</v>
       </c>
       <c r="B132" s="1" t="s">
-        <v>280</v>
+        <v>276</v>
       </c>
       <c r="C132" s="4" t="s">
-        <v>281</v>
+        <v>277</v>
       </c>
       <c r="D132" s="5">
-        <v>2.9</v>
+        <v>2.8</v>
       </c>
       <c r="E132" s="1"/>
       <c r="F132" s="1" t="s">
         <v>261</v>
       </c>
       <c r="G132" s="1" t="s">
-        <v>281</v>
+        <v>837</v>
       </c>
       <c r="H132" s="1" t="s">
         <v>12</v>
@@ -5637,45 +5646,45 @@
         <v>249</v>
       </c>
       <c r="B133" s="1" t="s">
-        <v>282</v>
+        <v>299</v>
       </c>
       <c r="C133" s="4" t="s">
-        <v>283</v>
+        <v>300</v>
       </c>
       <c r="D133" s="5">
-        <v>3.3</v>
+        <v>2.8</v>
       </c>
       <c r="E133" s="1"/>
       <c r="F133" s="1" t="s">
-        <v>264</v>
+        <v>252</v>
       </c>
       <c r="G133" s="1" t="s">
-        <v>283</v>
+        <v>301</v>
       </c>
       <c r="H133" s="1" t="s">
         <v>12</v>
       </c>
       <c r="I133" s="1"/>
     </row>
-    <row r="134" spans="1:9" ht="28.5">
+    <row r="134" spans="1:9">
       <c r="A134" s="1" t="s">
         <v>249</v>
       </c>
       <c r="B134" s="1" t="s">
-        <v>284</v>
+        <v>278</v>
       </c>
       <c r="C134" s="4" t="s">
-        <v>285</v>
+        <v>279</v>
       </c>
       <c r="D134" s="5">
-        <v>3</v>
+        <v>3.3</v>
       </c>
       <c r="E134" s="1"/>
       <c r="F134" s="1" t="s">
-        <v>261</v>
+        <v>252</v>
       </c>
       <c r="G134" s="1" t="s">
-        <v>285</v>
+        <v>279</v>
       </c>
       <c r="H134" s="1" t="s">
         <v>12</v>
@@ -5687,20 +5696,20 @@
         <v>249</v>
       </c>
       <c r="B135" s="1" t="s">
-        <v>286</v>
+        <v>280</v>
       </c>
       <c r="C135" s="4" t="s">
-        <v>287</v>
+        <v>281</v>
       </c>
       <c r="D135" s="5">
-        <v>3.2</v>
+        <v>2.9</v>
       </c>
       <c r="E135" s="1"/>
       <c r="F135" s="1" t="s">
-        <v>264</v>
+        <v>261</v>
       </c>
       <c r="G135" s="1" t="s">
-        <v>287</v>
+        <v>281</v>
       </c>
       <c r="H135" s="1" t="s">
         <v>12</v>
@@ -5712,42 +5721,46 @@
         <v>249</v>
       </c>
       <c r="B136" s="1" t="s">
-        <v>288</v>
+        <v>282</v>
       </c>
       <c r="C136" s="4" t="s">
-        <v>289</v>
+        <v>283</v>
       </c>
       <c r="D136" s="5">
-        <v>1.7</v>
+        <v>3.3</v>
       </c>
       <c r="E136" s="1"/>
       <c r="F136" s="1" t="s">
-        <v>257</v>
-      </c>
-      <c r="G136" s="1"/>
+        <v>264</v>
+      </c>
+      <c r="G136" s="1" t="s">
+        <v>283</v>
+      </c>
       <c r="H136" s="1" t="s">
         <v>12</v>
       </c>
       <c r="I136" s="1"/>
     </row>
-    <row r="137" spans="1:9">
+    <row r="137" spans="1:9" ht="28.5">
       <c r="A137" s="1" t="s">
         <v>249</v>
       </c>
       <c r="B137" s="1" t="s">
-        <v>290</v>
+        <v>284</v>
       </c>
       <c r="C137" s="4" t="s">
-        <v>291</v>
+        <v>285</v>
       </c>
       <c r="D137" s="5">
-        <v>2.2000000000000002</v>
+        <v>3</v>
       </c>
       <c r="E137" s="1"/>
       <c r="F137" s="1" t="s">
         <v>261</v>
       </c>
-      <c r="G137" s="1"/>
+      <c r="G137" s="1" t="s">
+        <v>285</v>
+      </c>
       <c r="H137" s="1" t="s">
         <v>12</v>
       </c>
@@ -5758,19 +5771,21 @@
         <v>249</v>
       </c>
       <c r="B138" s="1" t="s">
-        <v>292</v>
+        <v>286</v>
       </c>
       <c r="C138" s="4" t="s">
-        <v>293</v>
+        <v>287</v>
       </c>
       <c r="D138" s="5">
-        <v>2.5</v>
+        <v>3.2</v>
       </c>
       <c r="E138" s="1"/>
       <c r="F138" s="1" t="s">
         <v>264</v>
       </c>
-      <c r="G138" s="1"/>
+      <c r="G138" s="1" t="s">
+        <v>287</v>
+      </c>
       <c r="H138" s="1" t="s">
         <v>12</v>
       </c>
@@ -5781,21 +5796,19 @@
         <v>249</v>
       </c>
       <c r="B139" s="1" t="s">
-        <v>294</v>
+        <v>288</v>
       </c>
       <c r="C139" s="4" t="s">
-        <v>295</v>
+        <v>289</v>
       </c>
       <c r="D139" s="5">
-        <v>2.35</v>
+        <v>1.7</v>
       </c>
       <c r="E139" s="1"/>
       <c r="F139" s="1" t="s">
-        <v>261</v>
-      </c>
-      <c r="G139" s="1" t="s">
-        <v>296</v>
-      </c>
+        <v>257</v>
+      </c>
+      <c r="G139" s="1"/>
       <c r="H139" s="1" t="s">
         <v>12</v>
       </c>
@@ -5806,21 +5819,19 @@
         <v>249</v>
       </c>
       <c r="B140" s="1" t="s">
-        <v>297</v>
+        <v>290</v>
       </c>
       <c r="C140" s="4" t="s">
-        <v>298</v>
+        <v>291</v>
       </c>
       <c r="D140" s="5">
-        <v>2.2999999999999998</v>
+        <v>2.2000000000000002</v>
       </c>
       <c r="E140" s="1"/>
       <c r="F140" s="1" t="s">
-        <v>264</v>
-      </c>
-      <c r="G140" s="1" t="s">
-        <v>296</v>
-      </c>
+        <v>261</v>
+      </c>
+      <c r="G140" s="1"/>
       <c r="H140" s="1" t="s">
         <v>12</v>
       </c>
@@ -5831,21 +5842,19 @@
         <v>249</v>
       </c>
       <c r="B141" s="1" t="s">
-        <v>299</v>
+        <v>292</v>
       </c>
       <c r="C141" s="4" t="s">
-        <v>300</v>
+        <v>293</v>
       </c>
       <c r="D141" s="5">
-        <v>2.8</v>
+        <v>2.5</v>
       </c>
       <c r="E141" s="1"/>
       <c r="F141" s="1" t="s">
-        <v>252</v>
-      </c>
-      <c r="G141" s="1" t="s">
-        <v>301</v>
-      </c>
+        <v>264</v>
+      </c>
+      <c r="G141" s="1"/>
       <c r="H141" s="1" t="s">
         <v>12</v>
       </c>
@@ -5869,7 +5878,7 @@
         <v>252</v>
       </c>
       <c r="G142" s="1" t="s">
-        <v>304</v>
+        <v>838</v>
       </c>
       <c r="H142" s="1" t="s">
         <v>12</v>
@@ -5881,10 +5890,10 @@
         <v>249</v>
       </c>
       <c r="B143" s="1" t="s">
+        <v>304</v>
+      </c>
+      <c r="C143" s="4" t="s">
         <v>305</v>
-      </c>
-      <c r="C143" s="4" t="s">
-        <v>306</v>
       </c>
       <c r="D143" s="5">
         <v>2.5</v>
@@ -5894,7 +5903,7 @@
         <v>252</v>
       </c>
       <c r="G143" s="1" t="s">
-        <v>307</v>
+        <v>306</v>
       </c>
       <c r="H143" s="1" t="s">
         <v>12</v>
@@ -5903,13 +5912,13 @@
     </row>
     <row r="144" spans="1:9">
       <c r="A144" s="1" t="s">
+        <v>307</v>
+      </c>
+      <c r="B144" s="1" t="s">
         <v>308</v>
       </c>
-      <c r="B144" s="1" t="s">
+      <c r="C144" s="4" t="s">
         <v>309</v>
-      </c>
-      <c r="C144" s="4" t="s">
-        <v>310</v>
       </c>
       <c r="D144" s="5">
         <v>2</v>
@@ -5924,13 +5933,13 @@
     </row>
     <row r="145" spans="1:9">
       <c r="A145" s="1" t="s">
-        <v>308</v>
+        <v>307</v>
       </c>
       <c r="B145" s="1" t="s">
+        <v>310</v>
+      </c>
+      <c r="C145" s="4" t="s">
         <v>311</v>
-      </c>
-      <c r="C145" s="4" t="s">
-        <v>312</v>
       </c>
       <c r="D145" s="5">
         <v>0.7</v>
@@ -5945,13 +5954,13 @@
     </row>
     <row r="146" spans="1:9">
       <c r="A146" s="1" t="s">
-        <v>308</v>
+        <v>307</v>
       </c>
       <c r="B146" s="1" t="s">
+        <v>312</v>
+      </c>
+      <c r="C146" s="4" t="s">
         <v>313</v>
-      </c>
-      <c r="C146" s="4" t="s">
-        <v>314</v>
       </c>
       <c r="D146" s="5">
         <v>0.8</v>
@@ -5966,13 +5975,13 @@
     </row>
     <row r="147" spans="1:9">
       <c r="A147" s="1" t="s">
-        <v>308</v>
-      </c>
-      <c r="B147" s="1" t="s">
-        <v>315</v>
+        <v>307</v>
+      </c>
+      <c r="B147" s="1">
+        <v>967</v>
       </c>
       <c r="C147" s="4" t="s">
-        <v>316</v>
+        <v>314</v>
       </c>
       <c r="D147" s="5">
         <v>3.5</v>
@@ -5987,13 +5996,13 @@
     </row>
     <row r="148" spans="1:9">
       <c r="A148" s="1" t="s">
-        <v>308</v>
+        <v>307</v>
       </c>
       <c r="B148" s="1" t="s">
-        <v>317</v>
+        <v>315</v>
       </c>
       <c r="C148" s="4" t="s">
-        <v>318</v>
+        <v>316</v>
       </c>
       <c r="D148" s="5">
         <v>1</v>
@@ -6008,13 +6017,13 @@
     </row>
     <row r="149" spans="1:9">
       <c r="A149" s="1" t="s">
-        <v>308</v>
+        <v>307</v>
       </c>
       <c r="B149" s="1" t="s">
-        <v>319</v>
+        <v>317</v>
       </c>
       <c r="C149" s="4" t="s">
-        <v>320</v>
+        <v>318</v>
       </c>
       <c r="D149" s="5">
         <v>2.5</v>
@@ -6029,13 +6038,13 @@
     </row>
     <row r="150" spans="1:9">
       <c r="A150" s="1" t="s">
-        <v>308</v>
+        <v>307</v>
       </c>
       <c r="B150" s="1" t="s">
-        <v>321</v>
+        <v>319</v>
       </c>
       <c r="C150" s="4" t="s">
-        <v>322</v>
+        <v>320</v>
       </c>
       <c r="D150" s="5">
         <v>2.5</v>
@@ -6050,13 +6059,13 @@
     </row>
     <row r="151" spans="1:9">
       <c r="A151" s="1" t="s">
-        <v>308</v>
+        <v>307</v>
       </c>
       <c r="B151" s="1" t="s">
-        <v>323</v>
+        <v>321</v>
       </c>
       <c r="C151" s="4" t="s">
-        <v>324</v>
+        <v>322</v>
       </c>
       <c r="D151" s="5">
         <v>3.5</v>
@@ -6071,13 +6080,13 @@
     </row>
     <row r="152" spans="1:9">
       <c r="A152" s="1" t="s">
-        <v>308</v>
+        <v>307</v>
       </c>
       <c r="B152" s="1" t="s">
-        <v>325</v>
+        <v>323</v>
       </c>
       <c r="C152" s="4" t="s">
-        <v>326</v>
+        <v>324</v>
       </c>
       <c r="D152" s="5">
         <v>3.2</v>
@@ -6092,13 +6101,13 @@
     </row>
     <row r="153" spans="1:9">
       <c r="A153" s="1" t="s">
-        <v>308</v>
+        <v>307</v>
       </c>
       <c r="B153" s="1" t="s">
-        <v>327</v>
+        <v>325</v>
       </c>
       <c r="C153" s="4" t="s">
-        <v>328</v>
+        <v>326</v>
       </c>
       <c r="D153" s="5">
         <v>2</v>
@@ -6113,13 +6122,13 @@
     </row>
     <row r="154" spans="1:9">
       <c r="A154" s="1" t="s">
-        <v>308</v>
+        <v>307</v>
       </c>
       <c r="B154" s="1" t="s">
-        <v>329</v>
+        <v>327</v>
       </c>
       <c r="C154" s="4" t="s">
-        <v>330</v>
+        <v>328</v>
       </c>
       <c r="D154" s="5">
         <v>2</v>
@@ -6134,13 +6143,13 @@
     </row>
     <row r="155" spans="1:9">
       <c r="A155" s="1" t="s">
-        <v>308</v>
+        <v>307</v>
       </c>
       <c r="B155" s="1" t="s">
-        <v>331</v>
+        <v>329</v>
       </c>
       <c r="C155" s="4" t="s">
-        <v>332</v>
+        <v>330</v>
       </c>
       <c r="D155" s="5">
         <v>7.5</v>
@@ -6155,13 +6164,13 @@
     </row>
     <row r="156" spans="1:9">
       <c r="A156" s="1" t="s">
-        <v>308</v>
+        <v>307</v>
       </c>
       <c r="B156" s="1" t="s">
-        <v>333</v>
+        <v>331</v>
       </c>
       <c r="C156" s="4" t="s">
-        <v>334</v>
+        <v>332</v>
       </c>
       <c r="D156" s="5">
         <v>2</v>
@@ -6176,13 +6185,13 @@
     </row>
     <row r="157" spans="1:9">
       <c r="A157" s="1" t="s">
-        <v>308</v>
+        <v>307</v>
       </c>
       <c r="B157" s="1" t="s">
-        <v>335</v>
+        <v>333</v>
       </c>
       <c r="C157" s="4" t="s">
-        <v>336</v>
+        <v>334</v>
       </c>
       <c r="D157" s="5">
         <v>3</v>
@@ -6197,13 +6206,13 @@
     </row>
     <row r="158" spans="1:9">
       <c r="A158" s="1" t="s">
-        <v>308</v>
+        <v>307</v>
       </c>
       <c r="B158" s="1" t="s">
-        <v>337</v>
+        <v>335</v>
       </c>
       <c r="C158" s="4" t="s">
-        <v>338</v>
+        <v>336</v>
       </c>
       <c r="D158" s="5">
         <v>3.1</v>
@@ -6218,13 +6227,13 @@
     </row>
     <row r="159" spans="1:9">
       <c r="A159" s="1" t="s">
-        <v>308</v>
+        <v>307</v>
       </c>
       <c r="B159" s="1" t="s">
-        <v>339</v>
+        <v>337</v>
       </c>
       <c r="C159" s="4" t="s">
-        <v>340</v>
+        <v>338</v>
       </c>
       <c r="D159" s="5">
         <v>0.15</v>
@@ -6239,13 +6248,13 @@
     </row>
     <row r="160" spans="1:9">
       <c r="A160" s="1" t="s">
-        <v>308</v>
+        <v>307</v>
       </c>
       <c r="B160" s="1" t="s">
-        <v>341</v>
+        <v>339</v>
       </c>
       <c r="C160" s="4" t="s">
-        <v>342</v>
+        <v>340</v>
       </c>
       <c r="D160" s="5">
         <v>0.06</v>
@@ -6260,13 +6269,13 @@
     </row>
     <row r="161" spans="1:9">
       <c r="A161" s="1" t="s">
-        <v>308</v>
+        <v>307</v>
       </c>
       <c r="B161" s="1" t="s">
-        <v>343</v>
+        <v>341</v>
       </c>
       <c r="C161" s="4" t="s">
-        <v>344</v>
+        <v>342</v>
       </c>
       <c r="D161" s="5">
         <v>5.5</v>
@@ -6281,13 +6290,13 @@
     </row>
     <row r="162" spans="1:9">
       <c r="A162" s="1" t="s">
-        <v>308</v>
+        <v>307</v>
       </c>
       <c r="B162" s="1" t="s">
-        <v>345</v>
+        <v>343</v>
       </c>
       <c r="C162" s="4" t="s">
-        <v>346</v>
+        <v>344</v>
       </c>
       <c r="D162" s="5">
         <v>0.2</v>
@@ -6302,13 +6311,13 @@
     </row>
     <row r="163" spans="1:9">
       <c r="A163" s="1" t="s">
-        <v>308</v>
+        <v>307</v>
       </c>
       <c r="B163" s="1" t="s">
-        <v>347</v>
+        <v>345</v>
       </c>
       <c r="C163" s="4" t="s">
-        <v>348</v>
+        <v>346</v>
       </c>
       <c r="D163" s="5">
         <v>7.0000000000000007E-2</v>
@@ -6323,13 +6332,13 @@
     </row>
     <row r="164" spans="1:9">
       <c r="A164" s="1" t="s">
-        <v>308</v>
+        <v>307</v>
       </c>
       <c r="B164" s="1" t="s">
-        <v>349</v>
+        <v>347</v>
       </c>
       <c r="C164" s="4" t="s">
-        <v>350</v>
+        <v>348</v>
       </c>
       <c r="D164" s="5">
         <v>1</v>
@@ -6344,13 +6353,13 @@
     </row>
     <row r="165" spans="1:9">
       <c r="A165" s="1" t="s">
-        <v>308</v>
+        <v>307</v>
       </c>
       <c r="B165" s="1" t="s">
-        <v>351</v>
+        <v>349</v>
       </c>
       <c r="C165" s="4" t="s">
-        <v>352</v>
+        <v>350</v>
       </c>
       <c r="D165" s="5">
         <v>1.5</v>
@@ -6365,13 +6374,13 @@
     </row>
     <row r="166" spans="1:9">
       <c r="A166" s="1" t="s">
-        <v>308</v>
+        <v>307</v>
       </c>
       <c r="B166" s="1" t="s">
-        <v>353</v>
+        <v>351</v>
       </c>
       <c r="C166" s="4" t="s">
-        <v>354</v>
+        <v>352</v>
       </c>
       <c r="D166" s="5">
         <v>0.5</v>
@@ -6386,13 +6395,13 @@
     </row>
     <row r="167" spans="1:9">
       <c r="A167" s="1" t="s">
-        <v>308</v>
+        <v>307</v>
       </c>
       <c r="B167" s="1" t="s">
-        <v>355</v>
+        <v>353</v>
       </c>
       <c r="C167" s="4" t="s">
-        <v>356</v>
+        <v>354</v>
       </c>
       <c r="D167" s="5">
         <v>0.8</v>
@@ -6407,13 +6416,13 @@
     </row>
     <row r="168" spans="1:9">
       <c r="A168" s="1" t="s">
-        <v>308</v>
+        <v>307</v>
       </c>
       <c r="B168" s="1" t="s">
-        <v>357</v>
+        <v>355</v>
       </c>
       <c r="C168" s="4" t="s">
-        <v>358</v>
+        <v>356</v>
       </c>
       <c r="D168" s="5">
         <v>0.65</v>
@@ -6428,13 +6437,13 @@
     </row>
     <row r="169" spans="1:9">
       <c r="A169" s="1" t="s">
-        <v>308</v>
+        <v>307</v>
       </c>
       <c r="B169" s="1" t="s">
-        <v>359</v>
+        <v>357</v>
       </c>
       <c r="C169" s="4" t="s">
-        <v>360</v>
+        <v>358</v>
       </c>
       <c r="D169" s="5">
         <v>0.95</v>
@@ -6449,13 +6458,13 @@
     </row>
     <row r="170" spans="1:9">
       <c r="A170" s="1" t="s">
-        <v>308</v>
+        <v>307</v>
       </c>
       <c r="B170" s="1" t="s">
-        <v>361</v>
+        <v>359</v>
       </c>
       <c r="C170" s="4" t="s">
-        <v>362</v>
+        <v>360</v>
       </c>
       <c r="D170" s="5">
         <v>1.1000000000000001</v>
@@ -6470,13 +6479,13 @@
     </row>
     <row r="171" spans="1:9">
       <c r="A171" s="1" t="s">
-        <v>308</v>
+        <v>307</v>
       </c>
       <c r="B171" s="1" t="s">
-        <v>363</v>
+        <v>361</v>
       </c>
       <c r="C171" s="4" t="s">
-        <v>364</v>
+        <v>362</v>
       </c>
       <c r="D171" s="5">
         <v>2.1</v>
@@ -6491,13 +6500,13 @@
     </row>
     <row r="172" spans="1:9">
       <c r="A172" s="1" t="s">
-        <v>308</v>
+        <v>307</v>
       </c>
       <c r="B172" s="1" t="s">
-        <v>365</v>
+        <v>363</v>
       </c>
       <c r="C172" s="4" t="s">
-        <v>366</v>
+        <v>364</v>
       </c>
       <c r="D172" s="5">
         <v>1.5</v>
@@ -6512,13 +6521,13 @@
     </row>
     <row r="173" spans="1:9">
       <c r="A173" s="1" t="s">
-        <v>308</v>
+        <v>307</v>
       </c>
       <c r="B173" s="1" t="s">
-        <v>367</v>
+        <v>365</v>
       </c>
       <c r="C173" s="4" t="s">
-        <v>368</v>
+        <v>366</v>
       </c>
       <c r="D173" s="5">
         <v>0.4</v>
@@ -6533,13 +6542,13 @@
     </row>
     <row r="174" spans="1:9">
       <c r="A174" s="1" t="s">
-        <v>308</v>
+        <v>307</v>
       </c>
       <c r="B174" s="1" t="s">
-        <v>369</v>
+        <v>367</v>
       </c>
       <c r="C174" s="4" t="s">
-        <v>370</v>
+        <v>368</v>
       </c>
       <c r="D174" s="5">
         <v>0.6</v>
@@ -6554,13 +6563,13 @@
     </row>
     <row r="175" spans="1:9">
       <c r="A175" s="1" t="s">
+        <v>369</v>
+      </c>
+      <c r="B175" s="1" t="s">
+        <v>370</v>
+      </c>
+      <c r="C175" s="4" t="s">
         <v>371</v>
-      </c>
-      <c r="B175" s="1" t="s">
-        <v>372</v>
-      </c>
-      <c r="C175" s="4" t="s">
-        <v>373</v>
       </c>
       <c r="D175" s="5">
         <v>1</v>
@@ -6575,13 +6584,13 @@
     </row>
     <row r="176" spans="1:9">
       <c r="A176" s="1" t="s">
-        <v>371</v>
+        <v>369</v>
       </c>
       <c r="B176" s="1" t="s">
-        <v>374</v>
+        <v>372</v>
       </c>
       <c r="C176" s="4" t="s">
-        <v>375</v>
+        <v>373</v>
       </c>
       <c r="D176" s="5">
         <v>1</v>
@@ -6596,13 +6605,13 @@
     </row>
     <row r="177" spans="1:9">
       <c r="A177" s="1" t="s">
-        <v>371</v>
+        <v>369</v>
       </c>
       <c r="B177" s="1" t="s">
-        <v>376</v>
+        <v>374</v>
       </c>
       <c r="C177" s="4" t="s">
-        <v>377</v>
+        <v>375</v>
       </c>
       <c r="D177" s="5">
         <v>1.2</v>
@@ -6617,13 +6626,13 @@
     </row>
     <row r="178" spans="1:9">
       <c r="A178" s="1" t="s">
-        <v>371</v>
+        <v>369</v>
       </c>
       <c r="B178" s="1" t="s">
-        <v>378</v>
+        <v>376</v>
       </c>
       <c r="C178" s="4" t="s">
-        <v>379</v>
+        <v>377</v>
       </c>
       <c r="D178" s="5">
         <v>1.2</v>
@@ -6638,13 +6647,13 @@
     </row>
     <row r="179" spans="1:9">
       <c r="A179" s="1" t="s">
-        <v>371</v>
+        <v>369</v>
       </c>
       <c r="B179" s="1" t="s">
-        <v>380</v>
+        <v>378</v>
       </c>
       <c r="C179" s="4" t="s">
-        <v>381</v>
+        <v>379</v>
       </c>
       <c r="D179" s="5">
         <v>2</v>
@@ -6659,13 +6668,13 @@
     </row>
     <row r="180" spans="1:9">
       <c r="A180" s="1" t="s">
-        <v>371</v>
+        <v>369</v>
       </c>
       <c r="B180" s="1" t="s">
-        <v>382</v>
+        <v>380</v>
       </c>
       <c r="C180" s="4" t="s">
-        <v>383</v>
+        <v>381</v>
       </c>
       <c r="D180" s="5">
         <v>2.5</v>
@@ -6680,13 +6689,13 @@
     </row>
     <row r="181" spans="1:9">
       <c r="A181" s="1" t="s">
-        <v>371</v>
+        <v>369</v>
       </c>
       <c r="B181" s="1" t="s">
-        <v>384</v>
+        <v>382</v>
       </c>
       <c r="C181" s="4" t="s">
-        <v>385</v>
+        <v>383</v>
       </c>
       <c r="D181" s="5">
         <v>3.5</v>
@@ -6701,13 +6710,13 @@
     </row>
     <row r="182" spans="1:9">
       <c r="A182" s="1" t="s">
-        <v>371</v>
+        <v>369</v>
       </c>
       <c r="B182" s="1" t="s">
-        <v>386</v>
+        <v>384</v>
       </c>
       <c r="C182" s="4" t="s">
-        <v>387</v>
+        <v>385</v>
       </c>
       <c r="D182" s="5">
         <v>3.5</v>
@@ -6722,13 +6731,13 @@
     </row>
     <row r="183" spans="1:9">
       <c r="A183" s="1" t="s">
-        <v>371</v>
+        <v>369</v>
       </c>
       <c r="B183" s="1" t="s">
-        <v>388</v>
+        <v>386</v>
       </c>
       <c r="C183" s="4" t="s">
-        <v>389</v>
+        <v>387</v>
       </c>
       <c r="D183" s="5">
         <v>2.8</v>
@@ -6743,13 +6752,13 @@
     </row>
     <row r="184" spans="1:9">
       <c r="A184" s="1" t="s">
-        <v>371</v>
+        <v>369</v>
       </c>
       <c r="B184" s="1" t="s">
-        <v>390</v>
+        <v>388</v>
       </c>
       <c r="C184" s="4" t="s">
-        <v>391</v>
+        <v>389</v>
       </c>
       <c r="D184" s="5">
         <v>1.5</v>
@@ -6764,13 +6773,13 @@
     </row>
     <row r="185" spans="1:9">
       <c r="A185" s="1" t="s">
-        <v>371</v>
+        <v>369</v>
       </c>
       <c r="B185" s="1" t="s">
-        <v>392</v>
+        <v>390</v>
       </c>
       <c r="C185" s="4" t="s">
-        <v>393</v>
+        <v>391</v>
       </c>
       <c r="D185" s="5">
         <v>4.2</v>
@@ -6785,13 +6794,13 @@
     </row>
     <row r="186" spans="1:9">
       <c r="A186" s="1" t="s">
+        <v>392</v>
+      </c>
+      <c r="B186" s="1" t="s">
+        <v>393</v>
+      </c>
+      <c r="C186" s="4" t="s">
         <v>394</v>
-      </c>
-      <c r="B186" s="1" t="s">
-        <v>395</v>
-      </c>
-      <c r="C186" s="4" t="s">
-        <v>396</v>
       </c>
       <c r="D186" s="5">
         <v>1.2</v>
@@ -6806,13 +6815,13 @@
     </row>
     <row r="187" spans="1:9">
       <c r="A187" s="1" t="s">
-        <v>394</v>
+        <v>392</v>
       </c>
       <c r="B187" s="1" t="s">
-        <v>397</v>
+        <v>395</v>
       </c>
       <c r="C187" s="4" t="s">
-        <v>398</v>
+        <v>396</v>
       </c>
       <c r="D187" s="5">
         <v>1.2</v>
@@ -6827,13 +6836,13 @@
     </row>
     <row r="188" spans="1:9">
       <c r="A188" s="1" t="s">
-        <v>394</v>
+        <v>392</v>
       </c>
       <c r="B188" s="1" t="s">
-        <v>399</v>
+        <v>397</v>
       </c>
       <c r="C188" s="4" t="s">
-        <v>400</v>
+        <v>398</v>
       </c>
       <c r="D188" s="5">
         <v>1.2</v>
@@ -6848,13 +6857,13 @@
     </row>
     <row r="189" spans="1:9">
       <c r="A189" s="1" t="s">
-        <v>394</v>
+        <v>392</v>
       </c>
       <c r="B189" s="1" t="s">
-        <v>401</v>
+        <v>399</v>
       </c>
       <c r="C189" s="4" t="s">
-        <v>402</v>
+        <v>400</v>
       </c>
       <c r="D189" s="5">
         <v>2</v>
@@ -6869,13 +6878,13 @@
     </row>
     <row r="190" spans="1:9">
       <c r="A190" s="1" t="s">
-        <v>394</v>
+        <v>392</v>
       </c>
       <c r="B190" s="1" t="s">
-        <v>403</v>
+        <v>401</v>
       </c>
       <c r="C190" s="4" t="s">
-        <v>404</v>
+        <v>402</v>
       </c>
       <c r="D190" s="5">
         <v>1.2</v>
@@ -6890,13 +6899,13 @@
     </row>
     <row r="191" spans="1:9">
       <c r="A191" s="1" t="s">
-        <v>394</v>
+        <v>392</v>
       </c>
       <c r="B191" s="1" t="s">
-        <v>405</v>
+        <v>403</v>
       </c>
       <c r="C191" s="4" t="s">
-        <v>406</v>
+        <v>404</v>
       </c>
       <c r="D191" s="5">
         <v>2</v>
@@ -6911,13 +6920,13 @@
     </row>
     <row r="192" spans="1:9">
       <c r="A192" s="1" t="s">
-        <v>394</v>
+        <v>392</v>
       </c>
       <c r="B192" s="1" t="s">
-        <v>407</v>
+        <v>405</v>
       </c>
       <c r="C192" s="4" t="s">
-        <v>408</v>
+        <v>406</v>
       </c>
       <c r="D192" s="5">
         <v>6.5</v>
@@ -6932,13 +6941,13 @@
     </row>
     <row r="193" spans="1:9">
       <c r="A193" s="1" t="s">
-        <v>394</v>
+        <v>392</v>
       </c>
       <c r="B193" s="1" t="s">
-        <v>409</v>
+        <v>407</v>
       </c>
       <c r="C193" s="4" t="s">
-        <v>410</v>
+        <v>408</v>
       </c>
       <c r="D193" s="5">
         <v>1.2</v>
@@ -6953,13 +6962,13 @@
     </row>
     <row r="194" spans="1:9">
       <c r="A194" s="1" t="s">
-        <v>394</v>
+        <v>392</v>
       </c>
       <c r="B194" s="1" t="s">
-        <v>411</v>
+        <v>409</v>
       </c>
       <c r="C194" s="4" t="s">
-        <v>412</v>
+        <v>410</v>
       </c>
       <c r="D194" s="5">
         <v>1</v>
@@ -6974,13 +6983,13 @@
     </row>
     <row r="195" spans="1:9">
       <c r="A195" s="1" t="s">
-        <v>394</v>
+        <v>392</v>
       </c>
       <c r="B195" s="1" t="s">
-        <v>413</v>
+        <v>411</v>
       </c>
       <c r="C195" s="4" t="s">
-        <v>414</v>
+        <v>412</v>
       </c>
       <c r="D195" s="5">
         <v>1.3</v>
@@ -6995,13 +7004,13 @@
     </row>
     <row r="196" spans="1:9">
       <c r="A196" s="1" t="s">
-        <v>394</v>
+        <v>392</v>
       </c>
       <c r="B196" s="1" t="s">
-        <v>415</v>
+        <v>413</v>
       </c>
       <c r="C196" s="4" t="s">
-        <v>416</v>
+        <v>414</v>
       </c>
       <c r="D196" s="5">
         <v>0.2</v>
@@ -7016,13 +7025,13 @@
     </row>
     <row r="197" spans="1:9">
       <c r="A197" s="1" t="s">
-        <v>394</v>
+        <v>392</v>
       </c>
       <c r="B197" s="1" t="s">
-        <v>417</v>
+        <v>415</v>
       </c>
       <c r="C197" s="4" t="s">
-        <v>418</v>
+        <v>416</v>
       </c>
       <c r="D197" s="5">
         <v>1.5</v>
@@ -7037,13 +7046,13 @@
     </row>
     <row r="198" spans="1:9">
       <c r="A198" s="1" t="s">
-        <v>394</v>
+        <v>392</v>
       </c>
       <c r="B198" s="1" t="s">
-        <v>419</v>
+        <v>417</v>
       </c>
       <c r="C198" s="4" t="s">
-        <v>420</v>
+        <v>418</v>
       </c>
       <c r="D198" s="5">
         <v>2</v>
@@ -7058,13 +7067,13 @@
     </row>
     <row r="199" spans="1:9">
       <c r="A199" s="1" t="s">
-        <v>394</v>
+        <v>392</v>
       </c>
       <c r="B199" s="1" t="s">
-        <v>421</v>
+        <v>419</v>
       </c>
       <c r="C199" s="4" t="s">
-        <v>422</v>
+        <v>420</v>
       </c>
       <c r="D199" s="5">
         <v>6</v>
@@ -7079,13 +7088,13 @@
     </row>
     <row r="200" spans="1:9">
       <c r="A200" s="1" t="s">
-        <v>394</v>
+        <v>392</v>
       </c>
       <c r="B200" s="1" t="s">
-        <v>423</v>
+        <v>421</v>
       </c>
       <c r="C200" s="4" t="s">
-        <v>424</v>
+        <v>422</v>
       </c>
       <c r="D200" s="5">
         <v>7</v>
@@ -7100,13 +7109,13 @@
     </row>
     <row r="201" spans="1:9">
       <c r="A201" s="1" t="s">
-        <v>394</v>
+        <v>392</v>
       </c>
       <c r="B201" s="1" t="s">
-        <v>425</v>
+        <v>423</v>
       </c>
       <c r="C201" s="4" t="s">
-        <v>426</v>
+        <v>424</v>
       </c>
       <c r="D201" s="5">
         <v>0.5</v>
@@ -7121,13 +7130,13 @@
     </row>
     <row r="202" spans="1:9">
       <c r="A202" s="1" t="s">
-        <v>394</v>
+        <v>392</v>
       </c>
       <c r="B202" s="1" t="s">
-        <v>427</v>
+        <v>425</v>
       </c>
       <c r="C202" s="4" t="s">
-        <v>428</v>
+        <v>426</v>
       </c>
       <c r="D202" s="5">
         <v>2.5</v>
@@ -7142,13 +7151,13 @@
     </row>
     <row r="203" spans="1:9">
       <c r="A203" s="1" t="s">
-        <v>394</v>
+        <v>392</v>
       </c>
       <c r="B203" s="1" t="s">
-        <v>429</v>
+        <v>427</v>
       </c>
       <c r="C203" s="4" t="s">
-        <v>430</v>
+        <v>428</v>
       </c>
       <c r="D203" s="5">
         <v>1</v>
@@ -7163,13 +7172,13 @@
     </row>
     <row r="204" spans="1:9">
       <c r="A204" s="1" t="s">
-        <v>394</v>
+        <v>392</v>
       </c>
       <c r="B204" s="1" t="s">
-        <v>431</v>
+        <v>429</v>
       </c>
       <c r="C204" s="4" t="s">
-        <v>432</v>
+        <v>430</v>
       </c>
       <c r="D204" s="5">
         <v>0.7</v>
@@ -7184,13 +7193,13 @@
     </row>
     <row r="205" spans="1:9">
       <c r="A205" s="1" t="s">
-        <v>394</v>
+        <v>392</v>
       </c>
       <c r="B205" s="1" t="s">
-        <v>433</v>
+        <v>431</v>
       </c>
       <c r="C205" s="4" t="s">
-        <v>434</v>
+        <v>432</v>
       </c>
       <c r="D205" s="5">
         <v>0.6</v>
@@ -7205,13 +7214,13 @@
     </row>
     <row r="206" spans="1:9">
       <c r="A206" s="1" t="s">
-        <v>394</v>
+        <v>392</v>
       </c>
       <c r="B206" s="1" t="s">
-        <v>435</v>
+        <v>433</v>
       </c>
       <c r="C206" s="4" t="s">
-        <v>436</v>
+        <v>434</v>
       </c>
       <c r="D206" s="5">
         <v>8</v>
@@ -7226,13 +7235,13 @@
     </row>
     <row r="207" spans="1:9">
       <c r="A207" s="1" t="s">
-        <v>394</v>
+        <v>392</v>
       </c>
       <c r="B207" s="1" t="s">
-        <v>437</v>
+        <v>435</v>
       </c>
       <c r="C207" s="4" t="s">
-        <v>438</v>
+        <v>436</v>
       </c>
       <c r="D207" s="5">
         <v>6.5</v>
@@ -7247,13 +7256,13 @@
     </row>
     <row r="208" spans="1:9">
       <c r="A208" s="1" t="s">
-        <v>394</v>
+        <v>392</v>
       </c>
       <c r="B208" s="1" t="s">
-        <v>439</v>
+        <v>437</v>
       </c>
       <c r="C208" s="4" t="s">
-        <v>440</v>
+        <v>438</v>
       </c>
       <c r="D208" s="5">
         <v>3</v>
@@ -7268,13 +7277,13 @@
     </row>
     <row r="209" spans="1:9">
       <c r="A209" s="1" t="s">
-        <v>394</v>
+        <v>392</v>
       </c>
       <c r="B209" s="1" t="s">
-        <v>441</v>
+        <v>439</v>
       </c>
       <c r="C209" s="4" t="s">
-        <v>442</v>
+        <v>440</v>
       </c>
       <c r="D209" s="5">
         <v>4.5</v>
@@ -7289,13 +7298,13 @@
     </row>
     <row r="210" spans="1:9">
       <c r="A210" s="1" t="s">
-        <v>394</v>
+        <v>392</v>
       </c>
       <c r="B210" s="1" t="s">
-        <v>443</v>
+        <v>441</v>
       </c>
       <c r="C210" s="4" t="s">
-        <v>444</v>
+        <v>442</v>
       </c>
       <c r="D210" s="5">
         <v>0.5</v>
@@ -7310,13 +7319,13 @@
     </row>
     <row r="211" spans="1:9">
       <c r="A211" s="1" t="s">
-        <v>394</v>
+        <v>392</v>
       </c>
       <c r="B211" s="1" t="s">
-        <v>445</v>
+        <v>443</v>
       </c>
       <c r="C211" s="4" t="s">
-        <v>446</v>
+        <v>444</v>
       </c>
       <c r="D211" s="5">
         <v>1.2</v>
@@ -7331,13 +7340,13 @@
     </row>
     <row r="212" spans="1:9">
       <c r="A212" s="1" t="s">
-        <v>394</v>
+        <v>392</v>
       </c>
       <c r="B212" s="1" t="s">
-        <v>447</v>
+        <v>445</v>
       </c>
       <c r="C212" s="4" t="s">
-        <v>448</v>
+        <v>446</v>
       </c>
       <c r="D212" s="5">
         <v>1.5</v>
@@ -7352,13 +7361,13 @@
     </row>
     <row r="213" spans="1:9">
       <c r="A213" s="1" t="s">
-        <v>394</v>
+        <v>392</v>
       </c>
       <c r="B213" s="1" t="s">
-        <v>449</v>
+        <v>447</v>
       </c>
       <c r="C213" s="4" t="s">
-        <v>450</v>
+        <v>448</v>
       </c>
       <c r="D213" s="5">
         <v>1.4</v>
@@ -7373,13 +7382,13 @@
     </row>
     <row r="214" spans="1:9">
       <c r="A214" s="1" t="s">
-        <v>394</v>
+        <v>392</v>
       </c>
       <c r="B214" s="1" t="s">
-        <v>451</v>
+        <v>449</v>
       </c>
       <c r="C214" s="4" t="s">
-        <v>452</v>
+        <v>450</v>
       </c>
       <c r="D214" s="5">
         <v>1.8</v>
@@ -7394,13 +7403,13 @@
     </row>
     <row r="215" spans="1:9">
       <c r="A215" s="1" t="s">
-        <v>394</v>
+        <v>392</v>
       </c>
       <c r="B215" s="1" t="s">
-        <v>453</v>
+        <v>451</v>
       </c>
       <c r="C215" s="4" t="s">
-        <v>454</v>
+        <v>452</v>
       </c>
       <c r="D215" s="5">
         <v>1.7</v>
@@ -7415,13 +7424,13 @@
     </row>
     <row r="216" spans="1:9">
       <c r="A216" s="1" t="s">
-        <v>394</v>
+        <v>392</v>
       </c>
       <c r="B216" s="1" t="s">
-        <v>455</v>
+        <v>453</v>
       </c>
       <c r="C216" s="4" t="s">
-        <v>456</v>
+        <v>454</v>
       </c>
       <c r="D216" s="5">
         <v>2.7</v>
@@ -7436,13 +7445,13 @@
     </row>
     <row r="217" spans="1:9">
       <c r="A217" s="1" t="s">
-        <v>394</v>
+        <v>392</v>
       </c>
       <c r="B217" s="1" t="s">
-        <v>457</v>
+        <v>455</v>
       </c>
       <c r="C217" s="4" t="s">
-        <v>458</v>
+        <v>456</v>
       </c>
       <c r="D217" s="5">
         <v>2.7</v>
@@ -7457,13 +7466,13 @@
     </row>
     <row r="218" spans="1:9">
       <c r="A218" s="1" t="s">
-        <v>394</v>
+        <v>392</v>
       </c>
       <c r="B218" s="1" t="s">
-        <v>459</v>
+        <v>457</v>
       </c>
       <c r="C218" s="4" t="s">
-        <v>460</v>
+        <v>458</v>
       </c>
       <c r="D218" s="5">
         <v>3.7</v>
@@ -7478,13 +7487,13 @@
     </row>
     <row r="219" spans="1:9">
       <c r="A219" s="1" t="s">
-        <v>394</v>
+        <v>392</v>
       </c>
       <c r="B219" s="1" t="s">
-        <v>461</v>
+        <v>459</v>
       </c>
       <c r="C219" s="4" t="s">
-        <v>462</v>
+        <v>460</v>
       </c>
       <c r="D219" s="5">
         <v>3.6</v>
@@ -7499,13 +7508,13 @@
     </row>
     <row r="220" spans="1:9">
       <c r="A220" s="1" t="s">
-        <v>394</v>
+        <v>392</v>
       </c>
       <c r="B220" s="1" t="s">
-        <v>463</v>
+        <v>461</v>
       </c>
       <c r="C220" s="4" t="s">
-        <v>464</v>
+        <v>462</v>
       </c>
       <c r="D220" s="5">
         <v>5</v>
@@ -7520,13 +7529,13 @@
     </row>
     <row r="221" spans="1:9">
       <c r="A221" s="1" t="s">
-        <v>394</v>
+        <v>392</v>
       </c>
       <c r="B221" s="1" t="s">
-        <v>465</v>
+        <v>463</v>
       </c>
       <c r="C221" s="4" t="s">
-        <v>466</v>
+        <v>464</v>
       </c>
       <c r="D221" s="5">
         <v>5.2</v>
@@ -7541,13 +7550,13 @@
     </row>
     <row r="222" spans="1:9">
       <c r="A222" s="1" t="s">
-        <v>394</v>
+        <v>392</v>
       </c>
       <c r="B222" s="1" t="s">
-        <v>467</v>
+        <v>465</v>
       </c>
       <c r="C222" s="4" t="s">
-        <v>468</v>
+        <v>466</v>
       </c>
       <c r="D222" s="5">
         <v>5</v>
@@ -7562,13 +7571,13 @@
     </row>
     <row r="223" spans="1:9">
       <c r="A223" s="1" t="s">
-        <v>394</v>
+        <v>392</v>
       </c>
       <c r="B223" s="1" t="s">
-        <v>469</v>
+        <v>467</v>
       </c>
       <c r="C223" s="4" t="s">
-        <v>470</v>
+        <v>468</v>
       </c>
       <c r="D223" s="5">
         <v>7</v>
@@ -7583,13 +7592,13 @@
     </row>
     <row r="224" spans="1:9">
       <c r="A224" s="1" t="s">
-        <v>394</v>
+        <v>392</v>
       </c>
       <c r="B224" s="1" t="s">
-        <v>471</v>
+        <v>469</v>
       </c>
       <c r="C224" s="4" t="s">
-        <v>472</v>
+        <v>470</v>
       </c>
       <c r="D224" s="5">
         <v>0.7</v>
@@ -7604,13 +7613,13 @@
     </row>
     <row r="225" spans="1:9">
       <c r="A225" s="1" t="s">
-        <v>394</v>
+        <v>392</v>
       </c>
       <c r="B225" s="1" t="s">
-        <v>473</v>
+        <v>471</v>
       </c>
       <c r="C225" s="4" t="s">
-        <v>474</v>
+        <v>472</v>
       </c>
       <c r="D225" s="5">
         <v>1</v>
@@ -7625,13 +7634,13 @@
     </row>
     <row r="226" spans="1:9">
       <c r="A226" s="1" t="s">
-        <v>394</v>
+        <v>392</v>
       </c>
       <c r="B226" s="1" t="s">
-        <v>475</v>
+        <v>473</v>
       </c>
       <c r="C226" s="4" t="s">
-        <v>476</v>
+        <v>474</v>
       </c>
       <c r="D226" s="5">
         <v>0.9</v>
@@ -7646,13 +7655,13 @@
     </row>
     <row r="227" spans="1:9">
       <c r="A227" s="1" t="s">
-        <v>394</v>
+        <v>392</v>
       </c>
       <c r="B227" s="1" t="s">
-        <v>477</v>
+        <v>475</v>
       </c>
       <c r="C227" s="4" t="s">
-        <v>478</v>
+        <v>476</v>
       </c>
       <c r="D227" s="5">
         <v>1.3</v>
@@ -7667,13 +7676,13 @@
     </row>
     <row r="228" spans="1:9">
       <c r="A228" s="1" t="s">
-        <v>394</v>
+        <v>392</v>
       </c>
       <c r="B228" s="1" t="s">
-        <v>479</v>
+        <v>477</v>
       </c>
       <c r="C228" s="4" t="s">
-        <v>480</v>
+        <v>478</v>
       </c>
       <c r="D228" s="5">
         <v>0.9</v>
@@ -7688,13 +7697,13 @@
     </row>
     <row r="229" spans="1:9">
       <c r="A229" s="1" t="s">
-        <v>394</v>
+        <v>392</v>
       </c>
       <c r="B229" s="1" t="s">
-        <v>481</v>
+        <v>479</v>
       </c>
       <c r="C229" s="4" t="s">
-        <v>482</v>
+        <v>480</v>
       </c>
       <c r="D229" s="5">
         <v>1.5</v>
@@ -7709,13 +7718,13 @@
     </row>
     <row r="230" spans="1:9">
       <c r="A230" s="1" t="s">
-        <v>394</v>
+        <v>392</v>
       </c>
       <c r="B230" s="1" t="s">
-        <v>483</v>
+        <v>481</v>
       </c>
       <c r="C230" s="4" t="s">
-        <v>484</v>
+        <v>482</v>
       </c>
       <c r="D230" s="5">
         <v>1.6</v>
@@ -7730,13 +7739,13 @@
     </row>
     <row r="231" spans="1:9">
       <c r="A231" s="1" t="s">
-        <v>394</v>
+        <v>392</v>
       </c>
       <c r="B231" s="1" t="s">
-        <v>485</v>
+        <v>483</v>
       </c>
       <c r="C231" s="4" t="s">
-        <v>486</v>
+        <v>484</v>
       </c>
       <c r="D231" s="5">
         <v>1.8</v>
@@ -7751,13 +7760,13 @@
     </row>
     <row r="232" spans="1:9">
       <c r="A232" s="1" t="s">
+        <v>485</v>
+      </c>
+      <c r="B232" s="1" t="s">
+        <v>486</v>
+      </c>
+      <c r="C232" s="4" t="s">
         <v>487</v>
-      </c>
-      <c r="B232" s="1" t="s">
-        <v>488</v>
-      </c>
-      <c r="C232" s="4" t="s">
-        <v>489</v>
       </c>
       <c r="D232" s="5">
         <v>0.5</v>
@@ -7772,13 +7781,13 @@
     </row>
     <row r="233" spans="1:9">
       <c r="A233" s="1" t="s">
-        <v>487</v>
+        <v>485</v>
       </c>
       <c r="B233" s="1" t="s">
-        <v>490</v>
+        <v>488</v>
       </c>
       <c r="C233" s="4" t="s">
-        <v>491</v>
+        <v>489</v>
       </c>
       <c r="D233" s="5">
         <v>0.6</v>
@@ -7793,13 +7802,13 @@
     </row>
     <row r="234" spans="1:9">
       <c r="A234" s="1" t="s">
-        <v>487</v>
+        <v>485</v>
       </c>
       <c r="B234" s="1" t="s">
-        <v>492</v>
+        <v>490</v>
       </c>
       <c r="C234" s="4" t="s">
-        <v>493</v>
+        <v>491</v>
       </c>
       <c r="D234" s="5">
         <v>0.7</v>
@@ -7814,13 +7823,13 @@
     </row>
     <row r="235" spans="1:9">
       <c r="A235" s="1" t="s">
-        <v>487</v>
+        <v>485</v>
       </c>
       <c r="B235" s="1" t="s">
-        <v>494</v>
+        <v>492</v>
       </c>
       <c r="C235" s="4" t="s">
-        <v>495</v>
+        <v>493</v>
       </c>
       <c r="D235" s="5">
         <v>0.8</v>
@@ -7835,13 +7844,13 @@
     </row>
     <row r="236" spans="1:9">
       <c r="A236" s="1" t="s">
-        <v>487</v>
+        <v>485</v>
       </c>
       <c r="B236" s="1" t="s">
-        <v>496</v>
+        <v>494</v>
       </c>
       <c r="C236" s="4" t="s">
-        <v>497</v>
+        <v>495</v>
       </c>
       <c r="D236" s="5">
         <v>0.9</v>
@@ -7856,13 +7865,13 @@
     </row>
     <row r="237" spans="1:9">
       <c r="A237" s="1" t="s">
-        <v>487</v>
+        <v>485</v>
       </c>
       <c r="B237" s="1" t="s">
-        <v>498</v>
+        <v>496</v>
       </c>
       <c r="C237" s="4" t="s">
-        <v>499</v>
+        <v>497</v>
       </c>
       <c r="D237" s="5">
         <v>1</v>
@@ -7877,13 +7886,13 @@
     </row>
     <row r="238" spans="1:9">
       <c r="A238" s="1" t="s">
-        <v>487</v>
+        <v>485</v>
       </c>
       <c r="B238" s="1" t="s">
-        <v>500</v>
+        <v>498</v>
       </c>
       <c r="C238" s="4" t="s">
-        <v>501</v>
+        <v>499</v>
       </c>
       <c r="D238" s="5">
         <v>1.5</v>
@@ -7898,13 +7907,13 @@
     </row>
     <row r="239" spans="1:9">
       <c r="A239" s="1" t="s">
-        <v>487</v>
+        <v>485</v>
       </c>
       <c r="B239" s="1" t="s">
-        <v>502</v>
+        <v>500</v>
       </c>
       <c r="C239" s="4" t="s">
-        <v>503</v>
+        <v>501</v>
       </c>
       <c r="D239" s="5">
         <v>2.2000000000000002</v>
@@ -7919,13 +7928,13 @@
     </row>
     <row r="240" spans="1:9">
       <c r="A240" s="1" t="s">
-        <v>487</v>
+        <v>485</v>
       </c>
       <c r="B240" s="1" t="s">
-        <v>504</v>
+        <v>502</v>
       </c>
       <c r="C240" s="4" t="s">
-        <v>505</v>
+        <v>503</v>
       </c>
       <c r="D240" s="5">
         <v>2.7</v>
@@ -7940,13 +7949,13 @@
     </row>
     <row r="241" spans="1:9">
       <c r="A241" s="1" t="s">
-        <v>487</v>
+        <v>485</v>
       </c>
       <c r="B241" s="1" t="s">
-        <v>506</v>
+        <v>504</v>
       </c>
       <c r="C241" s="4" t="s">
-        <v>507</v>
+        <v>505</v>
       </c>
       <c r="D241" s="5">
         <v>3.2</v>
@@ -7961,13 +7970,13 @@
     </row>
     <row r="242" spans="1:9">
       <c r="A242" s="1" t="s">
-        <v>487</v>
+        <v>485</v>
       </c>
       <c r="B242" s="1" t="s">
-        <v>508</v>
+        <v>506</v>
       </c>
       <c r="C242" s="4" t="s">
-        <v>509</v>
+        <v>507</v>
       </c>
       <c r="D242" s="5">
         <v>0.5</v>
@@ -7982,13 +7991,13 @@
     </row>
     <row r="243" spans="1:9">
       <c r="A243" s="1" t="s">
-        <v>487</v>
+        <v>485</v>
       </c>
       <c r="B243" s="1" t="s">
-        <v>510</v>
+        <v>508</v>
       </c>
       <c r="C243" s="4" t="s">
-        <v>511</v>
+        <v>509</v>
       </c>
       <c r="D243" s="5">
         <v>0.6</v>
@@ -8003,13 +8012,13 @@
     </row>
     <row r="244" spans="1:9">
       <c r="A244" s="1" t="s">
-        <v>487</v>
+        <v>485</v>
       </c>
       <c r="B244" s="1" t="s">
-        <v>512</v>
+        <v>510</v>
       </c>
       <c r="C244" s="4" t="s">
-        <v>513</v>
+        <v>511</v>
       </c>
       <c r="D244" s="5">
         <v>0.7</v>
@@ -8024,13 +8033,13 @@
     </row>
     <row r="245" spans="1:9">
       <c r="A245" s="1" t="s">
-        <v>487</v>
+        <v>485</v>
       </c>
       <c r="B245" s="1" t="s">
-        <v>514</v>
+        <v>512</v>
       </c>
       <c r="C245" s="4" t="s">
-        <v>515</v>
+        <v>513</v>
       </c>
       <c r="D245" s="5">
         <v>0.5</v>
@@ -8045,13 +8054,13 @@
     </row>
     <row r="246" spans="1:9">
       <c r="A246" s="1" t="s">
-        <v>487</v>
+        <v>485</v>
       </c>
       <c r="B246" s="1" t="s">
-        <v>516</v>
+        <v>514</v>
       </c>
       <c r="C246" s="4" t="s">
-        <v>517</v>
+        <v>515</v>
       </c>
       <c r="D246" s="5">
         <v>0.6</v>
@@ -8066,13 +8075,13 @@
     </row>
     <row r="247" spans="1:9">
       <c r="A247" s="1" t="s">
-        <v>487</v>
+        <v>485</v>
       </c>
       <c r="B247" s="1" t="s">
-        <v>518</v>
+        <v>516</v>
       </c>
       <c r="C247" s="4" t="s">
-        <v>519</v>
+        <v>517</v>
       </c>
       <c r="D247" s="5">
         <v>0.7</v>
@@ -8087,13 +8096,13 @@
     </row>
     <row r="248" spans="1:9">
       <c r="A248" s="1" t="s">
-        <v>487</v>
+        <v>485</v>
       </c>
       <c r="B248" s="1" t="s">
-        <v>520</v>
+        <v>518</v>
       </c>
       <c r="C248" s="4" t="s">
-        <v>521</v>
+        <v>519</v>
       </c>
       <c r="D248" s="5">
         <v>0.9</v>
@@ -8108,13 +8117,13 @@
     </row>
     <row r="249" spans="1:9">
       <c r="A249" s="1" t="s">
-        <v>487</v>
+        <v>485</v>
       </c>
       <c r="B249" s="1" t="s">
-        <v>522</v>
+        <v>520</v>
       </c>
       <c r="C249" s="4" t="s">
-        <v>523</v>
+        <v>521</v>
       </c>
       <c r="D249" s="5">
         <v>1</v>
@@ -8129,13 +8138,13 @@
     </row>
     <row r="250" spans="1:9">
       <c r="A250" s="1" t="s">
-        <v>487</v>
+        <v>485</v>
       </c>
       <c r="B250" s="1" t="s">
-        <v>524</v>
+        <v>522</v>
       </c>
       <c r="C250" s="4" t="s">
-        <v>525</v>
+        <v>523</v>
       </c>
       <c r="D250" s="5">
         <v>2</v>
@@ -8150,13 +8159,13 @@
     </row>
     <row r="251" spans="1:9">
       <c r="A251" s="1" t="s">
-        <v>487</v>
+        <v>485</v>
       </c>
       <c r="B251" s="1" t="s">
-        <v>526</v>
+        <v>524</v>
       </c>
       <c r="C251" s="4" t="s">
-        <v>527</v>
+        <v>525</v>
       </c>
       <c r="D251" s="5">
         <v>2.5</v>
@@ -8171,13 +8180,13 @@
     </row>
     <row r="252" spans="1:9">
       <c r="A252" s="1" t="s">
-        <v>487</v>
+        <v>485</v>
       </c>
       <c r="B252" s="1" t="s">
-        <v>528</v>
+        <v>526</v>
       </c>
       <c r="C252" s="4" t="s">
-        <v>529</v>
+        <v>527</v>
       </c>
       <c r="D252" s="5">
         <v>3.2</v>
@@ -8192,13 +8201,13 @@
     </row>
     <row r="253" spans="1:9">
       <c r="A253" s="1" t="s">
-        <v>487</v>
+        <v>485</v>
       </c>
       <c r="B253" s="1" t="s">
-        <v>530</v>
+        <v>528</v>
       </c>
       <c r="C253" s="4" t="s">
-        <v>531</v>
+        <v>529</v>
       </c>
       <c r="D253" s="5">
         <v>0.25</v>
@@ -8213,13 +8222,13 @@
     </row>
     <row r="254" spans="1:9">
       <c r="A254" s="1" t="s">
-        <v>487</v>
+        <v>485</v>
       </c>
       <c r="B254" s="1" t="s">
-        <v>532</v>
+        <v>530</v>
       </c>
       <c r="C254" s="4" t="s">
-        <v>533</v>
+        <v>531</v>
       </c>
       <c r="D254" s="5">
         <v>0.3</v>
@@ -8234,13 +8243,13 @@
     </row>
     <row r="255" spans="1:9">
       <c r="A255" s="1" t="s">
-        <v>487</v>
+        <v>485</v>
       </c>
       <c r="B255" s="1" t="s">
-        <v>534</v>
+        <v>532</v>
       </c>
       <c r="C255" s="4" t="s">
-        <v>535</v>
+        <v>533</v>
       </c>
       <c r="D255" s="5">
         <v>0.35</v>
@@ -8255,13 +8264,13 @@
     </row>
     <row r="256" spans="1:9">
       <c r="A256" s="1" t="s">
-        <v>487</v>
+        <v>485</v>
       </c>
       <c r="B256" s="1" t="s">
-        <v>536</v>
+        <v>534</v>
       </c>
       <c r="C256" s="4" t="s">
-        <v>537</v>
+        <v>535</v>
       </c>
       <c r="D256" s="5">
         <v>0.25</v>
@@ -8276,13 +8285,13 @@
     </row>
     <row r="257" spans="1:9">
       <c r="A257" s="1" t="s">
-        <v>487</v>
+        <v>485</v>
       </c>
       <c r="B257" s="1" t="s">
-        <v>538</v>
+        <v>536</v>
       </c>
       <c r="C257" s="4" t="s">
-        <v>539</v>
+        <v>537</v>
       </c>
       <c r="D257" s="5">
         <v>0.3</v>
@@ -8297,13 +8306,13 @@
     </row>
     <row r="258" spans="1:9">
       <c r="A258" s="1" t="s">
-        <v>487</v>
+        <v>485</v>
       </c>
       <c r="B258" s="1" t="s">
-        <v>540</v>
+        <v>538</v>
       </c>
       <c r="C258" s="4" t="s">
-        <v>541</v>
+        <v>539</v>
       </c>
       <c r="D258" s="5">
         <v>0.3</v>
@@ -8318,13 +8327,13 @@
     </row>
     <row r="259" spans="1:9">
       <c r="A259" s="1" t="s">
-        <v>487</v>
+        <v>485</v>
       </c>
       <c r="B259" s="1" t="s">
-        <v>542</v>
+        <v>540</v>
       </c>
       <c r="C259" s="4" t="s">
-        <v>543</v>
+        <v>541</v>
       </c>
       <c r="D259" s="5">
         <v>3.2</v>
@@ -8339,13 +8348,13 @@
     </row>
     <row r="260" spans="1:9">
       <c r="A260" s="1" t="s">
-        <v>487</v>
+        <v>485</v>
       </c>
       <c r="B260" s="1" t="s">
-        <v>544</v>
+        <v>542</v>
       </c>
       <c r="C260" s="4" t="s">
-        <v>545</v>
+        <v>543</v>
       </c>
       <c r="D260" s="5">
         <v>3</v>
@@ -8360,13 +8369,13 @@
     </row>
     <row r="261" spans="1:9">
       <c r="A261" s="1" t="s">
-        <v>487</v>
+        <v>485</v>
       </c>
       <c r="B261" s="1" t="s">
-        <v>546</v>
+        <v>544</v>
       </c>
       <c r="C261" s="4" t="s">
-        <v>547</v>
+        <v>545</v>
       </c>
       <c r="D261" s="5">
         <v>3.5</v>
@@ -8381,13 +8390,13 @@
     </row>
     <row r="262" spans="1:9">
       <c r="A262" s="1" t="s">
-        <v>487</v>
+        <v>485</v>
       </c>
       <c r="B262" s="1" t="s">
-        <v>548</v>
+        <v>546</v>
       </c>
       <c r="C262" s="4" t="s">
-        <v>549</v>
+        <v>547</v>
       </c>
       <c r="D262" s="5">
         <v>4.5</v>
@@ -8402,13 +8411,13 @@
     </row>
     <row r="263" spans="1:9">
       <c r="A263" s="1" t="s">
-        <v>487</v>
+        <v>485</v>
       </c>
       <c r="B263" s="1" t="s">
-        <v>550</v>
+        <v>548</v>
       </c>
       <c r="C263" s="4" t="s">
-        <v>551</v>
+        <v>549</v>
       </c>
       <c r="D263" s="5">
         <v>5.5</v>
@@ -8423,13 +8432,13 @@
     </row>
     <row r="264" spans="1:9">
       <c r="A264" s="1" t="s">
-        <v>487</v>
+        <v>485</v>
       </c>
       <c r="B264" s="1" t="s">
-        <v>552</v>
+        <v>550</v>
       </c>
       <c r="C264" s="4" t="s">
-        <v>553</v>
+        <v>551</v>
       </c>
       <c r="D264" s="5">
         <v>6</v>
@@ -8444,13 +8453,13 @@
     </row>
     <row r="265" spans="1:9">
       <c r="A265" s="1" t="s">
+        <v>552</v>
+      </c>
+      <c r="B265" s="1" t="s">
+        <v>553</v>
+      </c>
+      <c r="C265" s="4" t="s">
         <v>554</v>
-      </c>
-      <c r="B265" s="1" t="s">
-        <v>555</v>
-      </c>
-      <c r="C265" s="4" t="s">
-        <v>556</v>
       </c>
       <c r="D265" s="5">
         <v>8</v>
@@ -8465,13 +8474,13 @@
     </row>
     <row r="266" spans="1:9">
       <c r="A266" s="1" t="s">
-        <v>554</v>
+        <v>552</v>
       </c>
       <c r="B266" s="1" t="s">
-        <v>557</v>
+        <v>555</v>
       </c>
       <c r="C266" s="4" t="s">
-        <v>558</v>
+        <v>556</v>
       </c>
       <c r="D266" s="5">
         <v>8.5</v>
@@ -8486,13 +8495,13 @@
     </row>
     <row r="267" spans="1:9">
       <c r="A267" s="1" t="s">
-        <v>554</v>
+        <v>552</v>
       </c>
       <c r="B267" s="1" t="s">
-        <v>559</v>
+        <v>557</v>
       </c>
       <c r="C267" s="4" t="s">
-        <v>560</v>
+        <v>558</v>
       </c>
       <c r="D267" s="5">
         <v>8.6</v>
@@ -8507,13 +8516,13 @@
     </row>
     <row r="268" spans="1:9">
       <c r="A268" s="1" t="s">
-        <v>554</v>
+        <v>552</v>
       </c>
       <c r="B268" s="1" t="s">
-        <v>561</v>
+        <v>559</v>
       </c>
       <c r="C268" s="4" t="s">
-        <v>562</v>
+        <v>560</v>
       </c>
       <c r="D268" s="5">
         <v>8.9</v>
@@ -8528,13 +8537,13 @@
     </row>
     <row r="269" spans="1:9">
       <c r="A269" s="1" t="s">
-        <v>554</v>
+        <v>552</v>
       </c>
       <c r="B269" s="1" t="s">
-        <v>563</v>
+        <v>561</v>
       </c>
       <c r="C269" s="4" t="s">
-        <v>564</v>
+        <v>562</v>
       </c>
       <c r="D269" s="5">
         <v>8.9</v>
@@ -8549,13 +8558,13 @@
     </row>
     <row r="270" spans="1:9">
       <c r="A270" s="1" t="s">
-        <v>554</v>
+        <v>552</v>
       </c>
       <c r="B270" s="1" t="s">
-        <v>565</v>
+        <v>563</v>
       </c>
       <c r="C270" s="4" t="s">
-        <v>566</v>
+        <v>564</v>
       </c>
       <c r="D270" s="5">
         <v>9</v>
@@ -8570,13 +8579,13 @@
     </row>
     <row r="271" spans="1:9">
       <c r="A271" s="1" t="s">
-        <v>554</v>
+        <v>552</v>
       </c>
       <c r="B271" s="1" t="s">
-        <v>567</v>
+        <v>565</v>
       </c>
       <c r="C271" s="4" t="s">
-        <v>568</v>
+        <v>566</v>
       </c>
       <c r="D271" s="5">
         <v>9.4</v>
@@ -8591,13 +8600,13 @@
     </row>
     <row r="272" spans="1:9">
       <c r="A272" s="1" t="s">
-        <v>554</v>
+        <v>552</v>
       </c>
       <c r="B272" s="1" t="s">
-        <v>569</v>
+        <v>567</v>
       </c>
       <c r="C272" s="4" t="s">
-        <v>570</v>
+        <v>568</v>
       </c>
       <c r="D272" s="5">
         <v>9.8000000000000007</v>
@@ -8612,13 +8621,13 @@
     </row>
     <row r="273" spans="1:9">
       <c r="A273" s="1" t="s">
-        <v>554</v>
+        <v>552</v>
       </c>
       <c r="B273" s="1" t="s">
-        <v>571</v>
+        <v>569</v>
       </c>
       <c r="C273" s="4" t="s">
-        <v>572</v>
+        <v>570</v>
       </c>
       <c r="D273" s="5">
         <v>10.199999999999999</v>
@@ -8633,13 +8642,13 @@
     </row>
     <row r="274" spans="1:9">
       <c r="A274" s="1" t="s">
-        <v>554</v>
+        <v>552</v>
       </c>
       <c r="B274" s="1" t="s">
-        <v>573</v>
+        <v>571</v>
       </c>
       <c r="C274" s="4" t="s">
-        <v>574</v>
+        <v>572</v>
       </c>
       <c r="D274" s="5">
         <v>4.5</v>
@@ -8654,13 +8663,13 @@
     </row>
     <row r="275" spans="1:9">
       <c r="A275" s="1" t="s">
-        <v>554</v>
+        <v>552</v>
       </c>
       <c r="B275" s="1" t="s">
-        <v>575</v>
+        <v>573</v>
       </c>
       <c r="C275" s="4" t="s">
-        <v>576</v>
+        <v>574</v>
       </c>
       <c r="D275" s="5">
         <v>5.2</v>
@@ -8675,13 +8684,13 @@
     </row>
     <row r="276" spans="1:9">
       <c r="A276" s="1" t="s">
-        <v>554</v>
+        <v>552</v>
       </c>
       <c r="B276" s="1" t="s">
-        <v>577</v>
+        <v>575</v>
       </c>
       <c r="C276" s="4" t="s">
-        <v>578</v>
+        <v>576</v>
       </c>
       <c r="D276" s="5">
         <v>4.5</v>
@@ -8696,13 +8705,13 @@
     </row>
     <row r="277" spans="1:9">
       <c r="A277" s="1" t="s">
-        <v>554</v>
+        <v>552</v>
       </c>
       <c r="B277" s="1" t="s">
-        <v>579</v>
+        <v>577</v>
       </c>
       <c r="C277" s="4" t="s">
-        <v>580</v>
+        <v>578</v>
       </c>
       <c r="D277" s="5">
         <v>4.9000000000000004</v>
@@ -8717,13 +8726,13 @@
     </row>
     <row r="278" spans="1:9">
       <c r="A278" s="1" t="s">
-        <v>554</v>
+        <v>552</v>
       </c>
       <c r="B278" s="1" t="s">
-        <v>581</v>
+        <v>579</v>
       </c>
       <c r="C278" s="4" t="s">
-        <v>582</v>
+        <v>580</v>
       </c>
       <c r="D278" s="5">
         <v>5.2</v>
@@ -8738,13 +8747,13 @@
     </row>
     <row r="279" spans="1:9">
       <c r="A279" s="1" t="s">
-        <v>554</v>
+        <v>552</v>
       </c>
       <c r="B279" s="1" t="s">
-        <v>583</v>
+        <v>581</v>
       </c>
       <c r="C279" s="4" t="s">
-        <v>584</v>
+        <v>582</v>
       </c>
       <c r="D279" s="5">
         <v>5.5</v>
@@ -8759,13 +8768,13 @@
     </row>
     <row r="280" spans="1:9">
       <c r="A280" s="1" t="s">
-        <v>554</v>
+        <v>552</v>
       </c>
       <c r="B280" s="1" t="s">
-        <v>585</v>
+        <v>583</v>
       </c>
       <c r="C280" s="4" t="s">
-        <v>586</v>
+        <v>584</v>
       </c>
       <c r="D280" s="5">
         <v>6</v>
@@ -8780,13 +8789,13 @@
     </row>
     <row r="281" spans="1:9">
       <c r="A281" s="1" t="s">
-        <v>554</v>
+        <v>552</v>
       </c>
       <c r="B281" s="1" t="s">
-        <v>587</v>
+        <v>585</v>
       </c>
       <c r="C281" s="4" t="s">
-        <v>588</v>
+        <v>586</v>
       </c>
       <c r="D281" s="5">
         <v>6.2</v>
@@ -8801,13 +8810,13 @@
     </row>
     <row r="282" spans="1:9">
       <c r="A282" s="1" t="s">
-        <v>554</v>
+        <v>552</v>
       </c>
       <c r="B282" s="1" t="s">
-        <v>589</v>
+        <v>587</v>
       </c>
       <c r="C282" s="4" t="s">
-        <v>590</v>
+        <v>588</v>
       </c>
       <c r="D282" s="5">
         <v>6.5</v>
@@ -8822,13 +8831,13 @@
     </row>
     <row r="283" spans="1:9">
       <c r="A283" s="1" t="s">
-        <v>554</v>
+        <v>552</v>
       </c>
       <c r="B283" s="1" t="s">
-        <v>591</v>
+        <v>589</v>
       </c>
       <c r="C283" s="4" t="s">
-        <v>592</v>
+        <v>590</v>
       </c>
       <c r="D283" s="5">
         <v>6.8</v>
@@ -8843,13 +8852,13 @@
     </row>
     <row r="284" spans="1:9">
       <c r="A284" s="1" t="s">
-        <v>554</v>
+        <v>552</v>
       </c>
       <c r="B284" s="1" t="s">
-        <v>593</v>
+        <v>591</v>
       </c>
       <c r="C284" s="4" t="s">
-        <v>594</v>
+        <v>592</v>
       </c>
       <c r="D284" s="5">
         <v>3</v>
@@ -8864,13 +8873,13 @@
     </row>
     <row r="285" spans="1:9">
       <c r="A285" s="1" t="s">
-        <v>554</v>
+        <v>552</v>
       </c>
       <c r="B285" s="1" t="s">
-        <v>595</v>
+        <v>593</v>
       </c>
       <c r="C285" s="4" t="s">
-        <v>596</v>
+        <v>594</v>
       </c>
       <c r="D285" s="5">
         <v>5.5</v>
@@ -8885,13 +8894,13 @@
     </row>
     <row r="286" spans="1:9">
       <c r="A286" s="1" t="s">
+        <v>595</v>
+      </c>
+      <c r="B286" s="1" t="s">
+        <v>596</v>
+      </c>
+      <c r="C286" s="4" t="s">
         <v>597</v>
-      </c>
-      <c r="B286" s="1" t="s">
-        <v>598</v>
-      </c>
-      <c r="C286" s="4" t="s">
-        <v>599</v>
       </c>
       <c r="D286" s="5">
         <v>10</v>
@@ -8906,13 +8915,13 @@
     </row>
     <row r="287" spans="1:9">
       <c r="A287" s="1" t="s">
-        <v>597</v>
+        <v>595</v>
       </c>
       <c r="B287" s="1" t="s">
-        <v>600</v>
+        <v>598</v>
       </c>
       <c r="C287" s="4" t="s">
-        <v>601</v>
+        <v>599</v>
       </c>
       <c r="D287" s="5">
         <v>10</v>
@@ -8927,13 +8936,13 @@
     </row>
     <row r="288" spans="1:9">
       <c r="A288" s="1" t="s">
-        <v>597</v>
+        <v>595</v>
       </c>
       <c r="B288" s="1" t="s">
-        <v>602</v>
+        <v>600</v>
       </c>
       <c r="C288" s="4" t="s">
-        <v>603</v>
+        <v>601</v>
       </c>
       <c r="D288" s="5">
         <v>28</v>
@@ -8948,13 +8957,13 @@
     </row>
     <row r="289" spans="1:9">
       <c r="A289" s="1" t="s">
-        <v>597</v>
+        <v>595</v>
       </c>
       <c r="B289" s="1" t="s">
-        <v>604</v>
+        <v>602</v>
       </c>
       <c r="C289" s="4" t="s">
-        <v>605</v>
+        <v>603</v>
       </c>
       <c r="D289" s="5"/>
       <c r="E289" s="1"/>
@@ -8967,13 +8976,13 @@
     </row>
     <row r="290" spans="1:9">
       <c r="A290" s="1" t="s">
-        <v>597</v>
+        <v>595</v>
       </c>
       <c r="B290" s="1" t="s">
-        <v>606</v>
+        <v>604</v>
       </c>
       <c r="C290" s="4" t="s">
-        <v>607</v>
+        <v>605</v>
       </c>
       <c r="D290" s="5">
         <v>9</v>
@@ -8988,13 +8997,13 @@
     </row>
     <row r="291" spans="1:9">
       <c r="A291" s="1" t="s">
-        <v>597</v>
+        <v>595</v>
       </c>
       <c r="B291" s="1" t="s">
-        <v>608</v>
+        <v>606</v>
       </c>
       <c r="C291" s="4" t="s">
-        <v>609</v>
+        <v>607</v>
       </c>
       <c r="D291" s="5">
         <v>15</v>
@@ -9009,13 +9018,13 @@
     </row>
     <row r="292" spans="1:9">
       <c r="A292" s="1" t="s">
-        <v>597</v>
+        <v>595</v>
       </c>
       <c r="B292" s="1" t="s">
-        <v>610</v>
+        <v>608</v>
       </c>
       <c r="C292" s="4" t="s">
-        <v>611</v>
+        <v>609</v>
       </c>
       <c r="D292" s="5">
         <v>5</v>
@@ -9030,13 +9039,13 @@
     </row>
     <row r="293" spans="1:9">
       <c r="A293" s="1" t="s">
-        <v>597</v>
+        <v>595</v>
       </c>
       <c r="B293" s="1" t="s">
-        <v>612</v>
+        <v>610</v>
       </c>
       <c r="C293" s="4" t="s">
-        <v>613</v>
+        <v>611</v>
       </c>
       <c r="D293" s="5">
         <v>65</v>
@@ -9051,13 +9060,13 @@
     </row>
     <row r="294" spans="1:9">
       <c r="A294" s="1" t="s">
-        <v>597</v>
+        <v>595</v>
       </c>
       <c r="B294" s="1" t="s">
-        <v>614</v>
+        <v>612</v>
       </c>
       <c r="C294" s="4" t="s">
-        <v>615</v>
+        <v>613</v>
       </c>
       <c r="D294" s="5">
         <v>30</v>
@@ -9072,13 +9081,13 @@
     </row>
     <row r="295" spans="1:9">
       <c r="A295" s="1" t="s">
-        <v>597</v>
+        <v>595</v>
       </c>
       <c r="B295" s="1" t="s">
-        <v>616</v>
+        <v>614</v>
       </c>
       <c r="C295" s="4" t="s">
-        <v>617</v>
+        <v>615</v>
       </c>
       <c r="D295" s="5">
         <v>28</v>
@@ -9093,13 +9102,13 @@
     </row>
     <row r="296" spans="1:9">
       <c r="A296" s="1" t="s">
-        <v>597</v>
+        <v>595</v>
       </c>
       <c r="B296" s="1" t="s">
-        <v>618</v>
+        <v>616</v>
       </c>
       <c r="C296" s="4" t="s">
-        <v>619</v>
+        <v>617</v>
       </c>
       <c r="D296" s="5">
         <v>32</v>
@@ -9114,13 +9123,13 @@
     </row>
     <row r="297" spans="1:9">
       <c r="A297" s="1" t="s">
-        <v>597</v>
+        <v>595</v>
       </c>
       <c r="B297" s="1" t="s">
-        <v>620</v>
+        <v>618</v>
       </c>
       <c r="C297" s="4" t="s">
-        <v>621</v>
+        <v>619</v>
       </c>
       <c r="D297" s="5">
         <v>24</v>
@@ -9135,13 +9144,13 @@
     </row>
     <row r="298" spans="1:9">
       <c r="A298" s="1" t="s">
-        <v>597</v>
+        <v>595</v>
       </c>
       <c r="B298" s="1" t="s">
-        <v>622</v>
+        <v>620</v>
       </c>
       <c r="C298" s="4" t="s">
-        <v>623</v>
+        <v>621</v>
       </c>
       <c r="D298" s="5">
         <v>12</v>
@@ -9156,13 +9165,13 @@
     </row>
     <row r="299" spans="1:9">
       <c r="A299" s="1" t="s">
-        <v>597</v>
+        <v>595</v>
       </c>
       <c r="B299" s="1" t="s">
-        <v>624</v>
+        <v>622</v>
       </c>
       <c r="C299" s="4" t="s">
-        <v>625</v>
+        <v>623</v>
       </c>
       <c r="D299" s="5">
         <v>6</v>
@@ -9177,13 +9186,13 @@
     </row>
     <row r="300" spans="1:9">
       <c r="A300" s="1" t="s">
-        <v>597</v>
+        <v>595</v>
       </c>
       <c r="B300" s="1" t="s">
-        <v>626</v>
+        <v>624</v>
       </c>
       <c r="C300" s="4" t="s">
-        <v>627</v>
+        <v>625</v>
       </c>
       <c r="D300" s="5">
         <v>3</v>
@@ -9198,13 +9207,13 @@
     </row>
     <row r="301" spans="1:9">
       <c r="A301" s="1" t="s">
+        <v>626</v>
+      </c>
+      <c r="B301" s="1" t="s">
+        <v>627</v>
+      </c>
+      <c r="C301" s="4" t="s">
         <v>628</v>
-      </c>
-      <c r="B301" s="1" t="s">
-        <v>629</v>
-      </c>
-      <c r="C301" s="4" t="s">
-        <v>630</v>
       </c>
       <c r="D301" s="5">
         <v>7.5</v>
@@ -9219,13 +9228,13 @@
     </row>
     <row r="302" spans="1:9">
       <c r="A302" s="1" t="s">
-        <v>628</v>
+        <v>626</v>
       </c>
       <c r="B302" s="1" t="s">
-        <v>631</v>
+        <v>629</v>
       </c>
       <c r="C302" s="4" t="s">
-        <v>632</v>
+        <v>630</v>
       </c>
       <c r="D302" s="5">
         <v>5</v>
@@ -9240,13 +9249,13 @@
     </row>
     <row r="303" spans="1:9">
       <c r="A303" s="1" t="s">
-        <v>628</v>
+        <v>626</v>
       </c>
       <c r="B303" s="1" t="s">
-        <v>633</v>
+        <v>631</v>
       </c>
       <c r="C303" s="4" t="s">
-        <v>634</v>
+        <v>632</v>
       </c>
       <c r="D303" s="5">
         <v>1</v>
@@ -9261,13 +9270,13 @@
     </row>
     <row r="304" spans="1:9">
       <c r="A304" s="1" t="s">
-        <v>628</v>
+        <v>626</v>
       </c>
       <c r="B304" s="1" t="s">
-        <v>635</v>
+        <v>633</v>
       </c>
       <c r="C304" s="4" t="s">
-        <v>636</v>
+        <v>634</v>
       </c>
       <c r="D304" s="5">
         <v>3</v>
@@ -9282,13 +9291,13 @@
     </row>
     <row r="305" spans="1:9">
       <c r="A305" s="1" t="s">
-        <v>628</v>
+        <v>626</v>
       </c>
       <c r="B305" s="1" t="s">
-        <v>637</v>
+        <v>635</v>
       </c>
       <c r="C305" s="4" t="s">
-        <v>638</v>
+        <v>636</v>
       </c>
       <c r="D305" s="5"/>
       <c r="E305" s="1"/>
@@ -9301,13 +9310,13 @@
     </row>
     <row r="306" spans="1:9">
       <c r="A306" s="1" t="s">
-        <v>628</v>
+        <v>626</v>
       </c>
       <c r="B306" s="1" t="s">
-        <v>639</v>
+        <v>637</v>
       </c>
       <c r="C306" s="4" t="s">
-        <v>640</v>
+        <v>638</v>
       </c>
       <c r="D306" s="5">
         <v>3.5</v>
@@ -9322,13 +9331,13 @@
     </row>
     <row r="307" spans="1:9">
       <c r="A307" s="1" t="s">
-        <v>628</v>
+        <v>626</v>
       </c>
       <c r="B307" s="1" t="s">
-        <v>641</v>
+        <v>639</v>
       </c>
       <c r="C307" s="4" t="s">
-        <v>642</v>
+        <v>640</v>
       </c>
       <c r="D307" s="5">
         <v>2.5</v>
@@ -9343,13 +9352,13 @@
     </row>
     <row r="308" spans="1:9">
       <c r="A308" s="1" t="s">
-        <v>628</v>
+        <v>626</v>
       </c>
       <c r="B308" s="1" t="s">
-        <v>643</v>
+        <v>641</v>
       </c>
       <c r="C308" s="4" t="s">
-        <v>644</v>
+        <v>642</v>
       </c>
       <c r="D308" s="5">
         <v>2.5</v>
@@ -9364,13 +9373,13 @@
     </row>
     <row r="309" spans="1:9">
       <c r="A309" s="1" t="s">
-        <v>628</v>
+        <v>626</v>
       </c>
       <c r="B309" s="1" t="s">
-        <v>645</v>
+        <v>643</v>
       </c>
       <c r="C309" s="4" t="s">
-        <v>646</v>
+        <v>644</v>
       </c>
       <c r="D309" s="5">
         <v>2.5</v>
@@ -9385,13 +9394,13 @@
     </row>
     <row r="310" spans="1:9">
       <c r="A310" s="1" t="s">
-        <v>628</v>
+        <v>626</v>
       </c>
       <c r="B310" s="1" t="s">
-        <v>647</v>
+        <v>645</v>
       </c>
       <c r="C310" s="4" t="s">
-        <v>648</v>
+        <v>646</v>
       </c>
       <c r="D310" s="5">
         <v>3.5</v>
@@ -9406,13 +9415,13 @@
     </row>
     <row r="311" spans="1:9">
       <c r="A311" s="1" t="s">
-        <v>628</v>
+        <v>626</v>
       </c>
       <c r="B311" s="1" t="s">
-        <v>649</v>
+        <v>647</v>
       </c>
       <c r="C311" s="4" t="s">
-        <v>650</v>
+        <v>648</v>
       </c>
       <c r="D311" s="5">
         <v>4.5</v>
@@ -9427,13 +9436,13 @@
     </row>
     <row r="312" spans="1:9">
       <c r="A312" s="1" t="s">
+        <v>649</v>
+      </c>
+      <c r="B312" s="1" t="s">
+        <v>650</v>
+      </c>
+      <c r="C312" s="4" t="s">
         <v>651</v>
-      </c>
-      <c r="B312" s="1" t="s">
-        <v>652</v>
-      </c>
-      <c r="C312" s="4" t="s">
-        <v>653</v>
       </c>
       <c r="D312" s="5">
         <v>6</v>
@@ -9448,13 +9457,13 @@
     </row>
     <row r="313" spans="1:9">
       <c r="A313" s="1" t="s">
-        <v>651</v>
+        <v>649</v>
       </c>
       <c r="B313" s="1" t="s">
-        <v>654</v>
+        <v>652</v>
       </c>
       <c r="C313" s="4" t="s">
-        <v>655</v>
+        <v>653</v>
       </c>
       <c r="D313" s="5">
         <v>3.5</v>
@@ -9469,13 +9478,13 @@
     </row>
     <row r="314" spans="1:9">
       <c r="A314" s="1" t="s">
-        <v>651</v>
+        <v>649</v>
       </c>
       <c r="B314" s="1" t="s">
-        <v>656</v>
+        <v>654</v>
       </c>
       <c r="C314" s="4" t="s">
-        <v>657</v>
+        <v>655</v>
       </c>
       <c r="D314" s="5">
         <v>15</v>
@@ -9490,13 +9499,13 @@
     </row>
     <row r="315" spans="1:9">
       <c r="A315" s="1" t="s">
-        <v>651</v>
+        <v>649</v>
       </c>
       <c r="B315" s="1" t="s">
-        <v>658</v>
+        <v>656</v>
       </c>
       <c r="C315" s="4" t="s">
-        <v>659</v>
+        <v>657</v>
       </c>
       <c r="D315" s="5">
         <v>4</v>
@@ -9511,13 +9520,13 @@
     </row>
     <row r="316" spans="1:9">
       <c r="A316" s="1" t="s">
+        <v>658</v>
+      </c>
+      <c r="B316" s="1" t="s">
+        <v>659</v>
+      </c>
+      <c r="C316" s="4" t="s">
         <v>660</v>
-      </c>
-      <c r="B316" s="1" t="s">
-        <v>661</v>
-      </c>
-      <c r="C316" s="4" t="s">
-        <v>662</v>
       </c>
       <c r="D316" s="5">
         <v>2</v>
@@ -9532,13 +9541,13 @@
     </row>
     <row r="317" spans="1:9">
       <c r="A317" s="1" t="s">
-        <v>660</v>
+        <v>658</v>
       </c>
       <c r="B317" s="1" t="s">
-        <v>663</v>
+        <v>661</v>
       </c>
       <c r="C317" s="4" t="s">
-        <v>664</v>
+        <v>662</v>
       </c>
       <c r="D317" s="5">
         <v>2</v>
@@ -9553,13 +9562,13 @@
     </row>
     <row r="318" spans="1:9">
       <c r="A318" s="1" t="s">
-        <v>660</v>
+        <v>658</v>
       </c>
       <c r="B318" s="1" t="s">
-        <v>665</v>
+        <v>663</v>
       </c>
       <c r="C318" s="4" t="s">
-        <v>666</v>
+        <v>664</v>
       </c>
       <c r="D318" s="5">
         <v>20</v>
@@ -9574,13 +9583,13 @@
     </row>
     <row r="319" spans="1:9">
       <c r="A319" s="1" t="s">
-        <v>660</v>
+        <v>658</v>
       </c>
       <c r="B319" s="1" t="s">
-        <v>667</v>
+        <v>665</v>
       </c>
       <c r="C319" s="4" t="s">
-        <v>668</v>
+        <v>666</v>
       </c>
       <c r="D319" s="5">
         <v>18</v>
@@ -9595,13 +9604,13 @@
     </row>
     <row r="320" spans="1:9">
       <c r="A320" s="1" t="s">
-        <v>660</v>
+        <v>658</v>
       </c>
       <c r="B320" s="1" t="s">
-        <v>669</v>
+        <v>667</v>
       </c>
       <c r="C320" s="4" t="s">
-        <v>670</v>
+        <v>668</v>
       </c>
       <c r="D320" s="5">
         <v>22</v>
@@ -9616,13 +9625,13 @@
     </row>
     <row r="321" spans="1:9">
       <c r="A321" s="1" t="s">
-        <v>660</v>
+        <v>658</v>
       </c>
       <c r="B321" s="1" t="s">
-        <v>671</v>
+        <v>669</v>
       </c>
       <c r="C321" s="4" t="s">
-        <v>672</v>
+        <v>670</v>
       </c>
       <c r="D321" s="5">
         <v>26</v>
@@ -9637,13 +9646,13 @@
     </row>
     <row r="322" spans="1:9">
       <c r="A322" s="1" t="s">
+        <v>671</v>
+      </c>
+      <c r="B322" s="1" t="s">
+        <v>672</v>
+      </c>
+      <c r="C322" s="4" t="s">
         <v>673</v>
-      </c>
-      <c r="B322" s="1" t="s">
-        <v>674</v>
-      </c>
-      <c r="C322" s="4" t="s">
-        <v>675</v>
       </c>
       <c r="D322" s="5">
         <v>0.25</v>
@@ -9658,13 +9667,13 @@
     </row>
     <row r="323" spans="1:9">
       <c r="A323" s="1" t="s">
-        <v>673</v>
+        <v>671</v>
       </c>
       <c r="B323" s="1" t="s">
-        <v>676</v>
+        <v>674</v>
       </c>
       <c r="C323" s="4" t="s">
-        <v>677</v>
+        <v>675</v>
       </c>
       <c r="D323" s="5">
         <v>0.6</v>
@@ -9679,13 +9688,13 @@
     </row>
     <row r="324" spans="1:9">
       <c r="A324" s="1" t="s">
-        <v>673</v>
+        <v>671</v>
       </c>
       <c r="B324" s="1" t="s">
-        <v>678</v>
+        <v>676</v>
       </c>
       <c r="C324" s="4" t="s">
-        <v>679</v>
+        <v>677</v>
       </c>
       <c r="D324" s="5">
         <v>0.8</v>
@@ -9700,13 +9709,13 @@
     </row>
     <row r="325" spans="1:9">
       <c r="A325" s="1" t="s">
-        <v>673</v>
+        <v>671</v>
       </c>
       <c r="B325" s="1" t="s">
-        <v>680</v>
+        <v>678</v>
       </c>
       <c r="C325" s="4" t="s">
-        <v>681</v>
+        <v>679</v>
       </c>
       <c r="D325" s="5">
         <v>0.6</v>
@@ -9721,13 +9730,13 @@
     </row>
     <row r="326" spans="1:9">
       <c r="A326" s="1" t="s">
-        <v>673</v>
+        <v>671</v>
       </c>
       <c r="B326" s="1" t="s">
-        <v>682</v>
+        <v>680</v>
       </c>
       <c r="C326" s="4" t="s">
-        <v>683</v>
+        <v>681</v>
       </c>
       <c r="D326" s="5">
         <v>0.8</v>
@@ -9742,13 +9751,13 @@
     </row>
     <row r="327" spans="1:9">
       <c r="A327" s="1" t="s">
-        <v>673</v>
+        <v>671</v>
       </c>
       <c r="B327" s="1" t="s">
-        <v>684</v>
+        <v>682</v>
       </c>
       <c r="C327" s="4" t="s">
-        <v>685</v>
+        <v>683</v>
       </c>
       <c r="D327" s="5">
         <v>1.5</v>
@@ -9763,13 +9772,13 @@
     </row>
     <row r="328" spans="1:9">
       <c r="A328" s="1" t="s">
-        <v>673</v>
+        <v>671</v>
       </c>
       <c r="B328" s="1" t="s">
-        <v>686</v>
+        <v>684</v>
       </c>
       <c r="C328" s="4" t="s">
-        <v>687</v>
+        <v>685</v>
       </c>
       <c r="D328" s="5">
         <v>2</v>
@@ -9784,13 +9793,13 @@
     </row>
     <row r="329" spans="1:9">
       <c r="A329" s="1" t="s">
-        <v>673</v>
+        <v>671</v>
       </c>
       <c r="B329" s="1" t="s">
-        <v>688</v>
+        <v>686</v>
       </c>
       <c r="C329" s="4" t="s">
-        <v>689</v>
+        <v>687</v>
       </c>
       <c r="D329" s="5">
         <v>2.5</v>
@@ -9805,13 +9814,13 @@
     </row>
     <row r="330" spans="1:9">
       <c r="A330" s="1" t="s">
-        <v>673</v>
+        <v>671</v>
       </c>
       <c r="B330" s="1" t="s">
-        <v>690</v>
+        <v>688</v>
       </c>
       <c r="C330" s="4" t="s">
-        <v>691</v>
+        <v>689</v>
       </c>
       <c r="D330" s="5">
         <v>1</v>
@@ -9826,13 +9835,13 @@
     </row>
     <row r="331" spans="1:9">
       <c r="A331" s="1" t="s">
-        <v>673</v>
+        <v>671</v>
       </c>
       <c r="B331" s="1" t="s">
-        <v>692</v>
+        <v>690</v>
       </c>
       <c r="C331" s="4" t="s">
-        <v>693</v>
+        <v>691</v>
       </c>
       <c r="D331" s="5">
         <v>0.1</v>
@@ -9847,13 +9856,13 @@
     </row>
     <row r="332" spans="1:9">
       <c r="A332" s="1" t="s">
-        <v>673</v>
+        <v>671</v>
       </c>
       <c r="B332" s="1" t="s">
-        <v>694</v>
+        <v>692</v>
       </c>
       <c r="C332" s="4" t="s">
-        <v>695</v>
+        <v>693</v>
       </c>
       <c r="D332" s="5">
         <v>0.5</v>
@@ -9868,13 +9877,13 @@
     </row>
     <row r="333" spans="1:9">
       <c r="A333" s="1" t="s">
-        <v>673</v>
+        <v>671</v>
       </c>
       <c r="B333" s="1" t="s">
-        <v>696</v>
+        <v>694</v>
       </c>
       <c r="C333" s="4" t="s">
-        <v>697</v>
+        <v>695</v>
       </c>
       <c r="D333" s="5">
         <v>1</v>
@@ -9889,13 +9898,13 @@
     </row>
     <row r="334" spans="1:9">
       <c r="A334" s="1" t="s">
-        <v>673</v>
+        <v>671</v>
       </c>
       <c r="B334" s="1" t="s">
-        <v>698</v>
+        <v>696</v>
       </c>
       <c r="C334" s="4" t="s">
-        <v>699</v>
+        <v>697</v>
       </c>
       <c r="D334" s="5">
         <v>0.5</v>
@@ -9910,13 +9919,13 @@
     </row>
     <row r="335" spans="1:9">
       <c r="A335" s="1" t="s">
-        <v>673</v>
+        <v>671</v>
       </c>
       <c r="B335" s="1" t="s">
-        <v>700</v>
+        <v>698</v>
       </c>
       <c r="C335" s="4" t="s">
-        <v>701</v>
+        <v>699</v>
       </c>
       <c r="D335" s="5">
         <v>0.5</v>
@@ -9931,13 +9940,13 @@
     </row>
     <row r="336" spans="1:9">
       <c r="A336" s="1" t="s">
-        <v>673</v>
+        <v>671</v>
       </c>
       <c r="B336" s="1" t="s">
-        <v>702</v>
+        <v>700</v>
       </c>
       <c r="C336" s="4" t="s">
-        <v>703</v>
+        <v>701</v>
       </c>
       <c r="D336" s="5">
         <v>1.2</v>
@@ -9952,13 +9961,13 @@
     </row>
     <row r="337" spans="1:9">
       <c r="A337" s="1" t="s">
-        <v>673</v>
+        <v>671</v>
       </c>
       <c r="B337" s="1" t="s">
-        <v>704</v>
+        <v>702</v>
       </c>
       <c r="C337" s="4" t="s">
-        <v>705</v>
+        <v>703</v>
       </c>
       <c r="D337" s="5">
         <v>1</v>
@@ -9973,13 +9982,13 @@
     </row>
     <row r="338" spans="1:9">
       <c r="A338" s="1" t="s">
+        <v>704</v>
+      </c>
+      <c r="B338" s="1" t="s">
+        <v>705</v>
+      </c>
+      <c r="C338" s="4" t="s">
         <v>706</v>
-      </c>
-      <c r="B338" s="1" t="s">
-        <v>707</v>
-      </c>
-      <c r="C338" s="4" t="s">
-        <v>708</v>
       </c>
       <c r="D338" s="5">
         <v>0.2</v>
@@ -9994,13 +10003,13 @@
     </row>
     <row r="339" spans="1:9">
       <c r="A339" s="1" t="s">
-        <v>706</v>
+        <v>704</v>
       </c>
       <c r="B339" s="1" t="s">
-        <v>709</v>
+        <v>707</v>
       </c>
       <c r="C339" s="4" t="s">
-        <v>710</v>
+        <v>708</v>
       </c>
       <c r="D339" s="5">
         <v>0.3</v>
@@ -10015,13 +10024,13 @@
     </row>
     <row r="340" spans="1:9">
       <c r="A340" s="1" t="s">
-        <v>706</v>
+        <v>704</v>
       </c>
       <c r="B340" s="1" t="s">
-        <v>711</v>
+        <v>709</v>
       </c>
       <c r="C340" s="4" t="s">
-        <v>712</v>
+        <v>710</v>
       </c>
       <c r="D340" s="5">
         <v>3</v>
@@ -10036,13 +10045,13 @@
     </row>
     <row r="341" spans="1:9">
       <c r="A341" s="1" t="s">
-        <v>706</v>
+        <v>704</v>
       </c>
       <c r="B341" s="1" t="s">
-        <v>713</v>
+        <v>711</v>
       </c>
       <c r="C341" s="4" t="s">
-        <v>714</v>
+        <v>712</v>
       </c>
       <c r="D341" s="5">
         <v>1</v>
@@ -10057,13 +10066,13 @@
     </row>
     <row r="342" spans="1:9">
       <c r="A342" s="1" t="s">
-        <v>706</v>
+        <v>704</v>
       </c>
       <c r="B342" s="1" t="s">
-        <v>715</v>
+        <v>713</v>
       </c>
       <c r="C342" s="4" t="s">
-        <v>716</v>
+        <v>714</v>
       </c>
       <c r="D342" s="5">
         <v>2</v>
@@ -10078,13 +10087,13 @@
     </row>
     <row r="343" spans="1:9">
       <c r="A343" s="1" t="s">
-        <v>706</v>
+        <v>704</v>
       </c>
       <c r="B343" s="1" t="s">
-        <v>717</v>
+        <v>715</v>
       </c>
       <c r="C343" s="4" t="s">
-        <v>718</v>
+        <v>716</v>
       </c>
       <c r="D343" s="5">
         <v>3.5</v>
@@ -10099,13 +10108,13 @@
     </row>
     <row r="344" spans="1:9">
       <c r="A344" s="1" t="s">
-        <v>706</v>
+        <v>704</v>
       </c>
       <c r="B344" s="1" t="s">
-        <v>719</v>
+        <v>717</v>
       </c>
       <c r="C344" s="4" t="s">
-        <v>720</v>
+        <v>718</v>
       </c>
       <c r="D344" s="5">
         <v>1.5</v>
@@ -10120,13 +10129,13 @@
     </row>
     <row r="345" spans="1:9">
       <c r="A345" s="1" t="s">
-        <v>706</v>
+        <v>704</v>
       </c>
       <c r="B345" s="1" t="s">
-        <v>721</v>
+        <v>719</v>
       </c>
       <c r="C345" s="4" t="s">
-        <v>722</v>
+        <v>720</v>
       </c>
       <c r="D345" s="5">
         <v>2.9</v>
@@ -10141,13 +10150,13 @@
     </row>
     <row r="346" spans="1:9">
       <c r="A346" s="1" t="s">
-        <v>706</v>
+        <v>704</v>
       </c>
       <c r="B346" s="1" t="s">
-        <v>723</v>
+        <v>721</v>
       </c>
       <c r="C346" s="4" t="s">
-        <v>724</v>
+        <v>722</v>
       </c>
       <c r="D346" s="5">
         <v>2.5</v>
@@ -10162,13 +10171,13 @@
     </row>
     <row r="347" spans="1:9">
       <c r="A347" s="1" t="s">
-        <v>706</v>
+        <v>704</v>
       </c>
       <c r="B347" s="1" t="s">
-        <v>725</v>
+        <v>723</v>
       </c>
       <c r="C347" s="4" t="s">
-        <v>726</v>
+        <v>724</v>
       </c>
       <c r="D347" s="5">
         <v>3</v>
@@ -10183,13 +10192,13 @@
     </row>
     <row r="348" spans="1:9">
       <c r="A348" s="1" t="s">
-        <v>706</v>
+        <v>704</v>
       </c>
       <c r="B348" s="1" t="s">
-        <v>727</v>
+        <v>725</v>
       </c>
       <c r="C348" s="4" t="s">
-        <v>728</v>
+        <v>726</v>
       </c>
       <c r="D348" s="5">
         <v>1.5</v>
@@ -10204,13 +10213,13 @@
     </row>
     <row r="349" spans="1:9">
       <c r="A349" s="1" t="s">
-        <v>706</v>
+        <v>704</v>
       </c>
       <c r="B349" s="1" t="s">
-        <v>729</v>
+        <v>727</v>
       </c>
       <c r="C349" s="4" t="s">
-        <v>730</v>
+        <v>728</v>
       </c>
       <c r="D349" s="5">
         <v>2.5</v>
@@ -10225,13 +10234,13 @@
     </row>
     <row r="350" spans="1:9">
       <c r="A350" s="1" t="s">
-        <v>706</v>
+        <v>704</v>
       </c>
       <c r="B350" s="1" t="s">
-        <v>731</v>
+        <v>729</v>
       </c>
       <c r="C350" s="4" t="s">
-        <v>732</v>
+        <v>730</v>
       </c>
       <c r="D350" s="5">
         <v>7.5</v>
@@ -10246,13 +10255,13 @@
     </row>
     <row r="351" spans="1:9">
       <c r="A351" s="1" t="s">
-        <v>706</v>
+        <v>704</v>
       </c>
       <c r="B351" s="1" t="s">
-        <v>733</v>
+        <v>731</v>
       </c>
       <c r="C351" s="4" t="s">
-        <v>734</v>
+        <v>732</v>
       </c>
       <c r="D351" s="5">
         <v>4.5</v>
@@ -10267,13 +10276,13 @@
     </row>
     <row r="352" spans="1:9">
       <c r="A352" s="1" t="s">
-        <v>706</v>
+        <v>704</v>
       </c>
       <c r="B352" s="1" t="s">
-        <v>735</v>
+        <v>733</v>
       </c>
       <c r="C352" s="4" t="s">
-        <v>736</v>
+        <v>734</v>
       </c>
       <c r="D352" s="5"/>
       <c r="E352" s="1"/>
@@ -10286,13 +10295,13 @@
     </row>
     <row r="353" spans="1:9">
       <c r="A353" s="1" t="s">
-        <v>706</v>
+        <v>704</v>
       </c>
       <c r="B353" s="1" t="s">
-        <v>737</v>
+        <v>735</v>
       </c>
       <c r="C353" s="4" t="s">
-        <v>738</v>
+        <v>736</v>
       </c>
       <c r="D353" s="5">
         <v>3</v>
@@ -10307,13 +10316,13 @@
     </row>
     <row r="354" spans="1:9">
       <c r="A354" s="1" t="s">
-        <v>706</v>
+        <v>704</v>
       </c>
       <c r="B354" s="1" t="s">
-        <v>739</v>
+        <v>737</v>
       </c>
       <c r="C354" s="4" t="s">
-        <v>740</v>
+        <v>738</v>
       </c>
       <c r="D354" s="5">
         <v>2</v>
@@ -10328,13 +10337,13 @@
     </row>
     <row r="355" spans="1:9">
       <c r="A355" s="1" t="s">
-        <v>706</v>
+        <v>704</v>
       </c>
       <c r="B355" s="1" t="s">
-        <v>741</v>
+        <v>739</v>
       </c>
       <c r="C355" s="4" t="s">
-        <v>742</v>
+        <v>740</v>
       </c>
       <c r="D355" s="5">
         <v>3</v>
@@ -10349,13 +10358,13 @@
     </row>
     <row r="356" spans="1:9">
       <c r="A356" s="1" t="s">
-        <v>706</v>
+        <v>704</v>
       </c>
       <c r="B356" s="1" t="s">
-        <v>743</v>
+        <v>741</v>
       </c>
       <c r="C356" s="4" t="s">
-        <v>744</v>
+        <v>742</v>
       </c>
       <c r="D356" s="5">
         <v>3</v>
@@ -10370,13 +10379,13 @@
     </row>
     <row r="357" spans="1:9">
       <c r="A357" s="1" t="s">
-        <v>706</v>
+        <v>704</v>
       </c>
       <c r="B357" s="1" t="s">
-        <v>745</v>
+        <v>743</v>
       </c>
       <c r="C357" s="4" t="s">
-        <v>746</v>
+        <v>744</v>
       </c>
       <c r="D357" s="5">
         <v>2</v>
@@ -10391,13 +10400,13 @@
     </row>
     <row r="358" spans="1:9">
       <c r="A358" s="1" t="s">
-        <v>706</v>
+        <v>704</v>
       </c>
       <c r="B358" s="1" t="s">
-        <v>747</v>
+        <v>745</v>
       </c>
       <c r="C358" s="4" t="s">
-        <v>748</v>
+        <v>746</v>
       </c>
       <c r="D358" s="5">
         <v>2</v>
@@ -10412,13 +10421,13 @@
     </row>
     <row r="359" spans="1:9">
       <c r="A359" s="1" t="s">
-        <v>706</v>
+        <v>704</v>
       </c>
       <c r="B359" s="1" t="s">
-        <v>749</v>
+        <v>747</v>
       </c>
       <c r="C359" s="4" t="s">
-        <v>750</v>
+        <v>748</v>
       </c>
       <c r="D359" s="5">
         <v>0.5</v>
@@ -10433,13 +10442,13 @@
     </row>
     <row r="360" spans="1:9">
       <c r="A360" s="1" t="s">
-        <v>706</v>
+        <v>704</v>
       </c>
       <c r="B360" s="1" t="s">
-        <v>751</v>
+        <v>749</v>
       </c>
       <c r="C360" s="4" t="s">
-        <v>752</v>
+        <v>750</v>
       </c>
       <c r="D360" s="5">
         <v>1</v>
@@ -10454,13 +10463,13 @@
     </row>
     <row r="361" spans="1:9">
       <c r="A361" s="1" t="s">
-        <v>706</v>
+        <v>704</v>
       </c>
       <c r="B361" s="1" t="s">
-        <v>753</v>
+        <v>751</v>
       </c>
       <c r="C361" s="4" t="s">
-        <v>754</v>
+        <v>752</v>
       </c>
       <c r="D361" s="5">
         <v>1</v>
@@ -10475,13 +10484,13 @@
     </row>
     <row r="362" spans="1:9">
       <c r="A362" s="1" t="s">
-        <v>706</v>
+        <v>704</v>
       </c>
       <c r="B362" s="1" t="s">
-        <v>755</v>
+        <v>753</v>
       </c>
       <c r="C362" s="4" t="s">
-        <v>756</v>
+        <v>754</v>
       </c>
       <c r="D362" s="5">
         <v>1</v>
@@ -10496,13 +10505,13 @@
     </row>
     <row r="363" spans="1:9">
       <c r="A363" s="1" t="s">
-        <v>706</v>
+        <v>704</v>
       </c>
       <c r="B363" s="1" t="s">
-        <v>757</v>
+        <v>755</v>
       </c>
       <c r="C363" s="4" t="s">
-        <v>758</v>
+        <v>756</v>
       </c>
       <c r="D363" s="5">
         <v>1</v>
@@ -10517,13 +10526,13 @@
     </row>
     <row r="364" spans="1:9">
       <c r="A364" s="1" t="s">
-        <v>706</v>
+        <v>704</v>
       </c>
       <c r="B364" s="1" t="s">
-        <v>759</v>
+        <v>757</v>
       </c>
       <c r="C364" s="4" t="s">
-        <v>760</v>
+        <v>758</v>
       </c>
       <c r="D364" s="5">
         <v>5.5</v>
@@ -10538,13 +10547,13 @@
     </row>
     <row r="365" spans="1:9">
       <c r="A365" s="1" t="s">
-        <v>706</v>
+        <v>704</v>
       </c>
       <c r="B365" s="1" t="s">
-        <v>761</v>
+        <v>759</v>
       </c>
       <c r="C365" s="4" t="s">
-        <v>762</v>
+        <v>760</v>
       </c>
       <c r="D365" s="5">
         <v>1.5</v>
@@ -10559,13 +10568,13 @@
     </row>
     <row r="366" spans="1:9">
       <c r="A366" s="1" t="s">
-        <v>706</v>
+        <v>704</v>
       </c>
       <c r="B366" s="1" t="s">
-        <v>763</v>
+        <v>761</v>
       </c>
       <c r="C366" s="4" t="s">
-        <v>764</v>
+        <v>762</v>
       </c>
       <c r="D366" s="5">
         <v>3</v>
@@ -10580,13 +10589,13 @@
     </row>
     <row r="367" spans="1:9">
       <c r="A367" s="1" t="s">
-        <v>706</v>
+        <v>704</v>
       </c>
       <c r="B367" s="1" t="s">
-        <v>765</v>
+        <v>763</v>
       </c>
       <c r="C367" s="4" t="s">
-        <v>766</v>
+        <v>764</v>
       </c>
       <c r="D367" s="5">
         <v>4.5</v>
@@ -10601,13 +10610,13 @@
     </row>
     <row r="368" spans="1:9">
       <c r="A368" s="1" t="s">
-        <v>706</v>
+        <v>704</v>
       </c>
       <c r="B368" s="1" t="s">
-        <v>767</v>
+        <v>765</v>
       </c>
       <c r="C368" s="4" t="s">
-        <v>768</v>
+        <v>766</v>
       </c>
       <c r="D368" s="5">
         <v>8</v>
@@ -10622,13 +10631,13 @@
     </row>
     <row r="369" spans="1:9">
       <c r="A369" s="1" t="s">
-        <v>706</v>
+        <v>704</v>
       </c>
       <c r="B369" s="1" t="s">
-        <v>769</v>
+        <v>767</v>
       </c>
       <c r="C369" s="4" t="s">
-        <v>770</v>
+        <v>768</v>
       </c>
       <c r="D369" s="5">
         <v>18</v>
@@ -10643,13 +10652,13 @@
     </row>
     <row r="370" spans="1:9">
       <c r="A370" s="1" t="s">
-        <v>706</v>
+        <v>704</v>
       </c>
       <c r="B370" s="1" t="s">
-        <v>771</v>
+        <v>769</v>
       </c>
       <c r="C370" s="4" t="s">
-        <v>772</v>
+        <v>770</v>
       </c>
       <c r="D370" s="5">
         <v>3</v>
@@ -10664,13 +10673,13 @@
     </row>
     <row r="371" spans="1:9">
       <c r="A371" s="1" t="s">
-        <v>706</v>
+        <v>704</v>
       </c>
       <c r="B371" s="1" t="s">
-        <v>773</v>
+        <v>771</v>
       </c>
       <c r="C371" s="4" t="s">
-        <v>774</v>
+        <v>772</v>
       </c>
       <c r="D371" s="5"/>
       <c r="E371" s="1"/>
@@ -10683,13 +10692,13 @@
     </row>
     <row r="372" spans="1:9">
       <c r="A372" s="1" t="s">
-        <v>706</v>
+        <v>704</v>
       </c>
       <c r="B372" s="1" t="s">
-        <v>775</v>
+        <v>773</v>
       </c>
       <c r="C372" s="4" t="s">
-        <v>776</v>
+        <v>774</v>
       </c>
       <c r="D372" s="5">
         <v>0.6</v>
@@ -10704,13 +10713,13 @@
     </row>
     <row r="373" spans="1:9">
       <c r="A373" s="1" t="s">
-        <v>706</v>
+        <v>704</v>
       </c>
       <c r="B373" s="1" t="s">
-        <v>777</v>
+        <v>775</v>
       </c>
       <c r="C373" s="4" t="s">
-        <v>778</v>
+        <v>776</v>
       </c>
       <c r="D373" s="5">
         <v>1.2</v>
@@ -10725,13 +10734,13 @@
     </row>
     <row r="374" spans="1:9">
       <c r="A374" s="1" t="s">
-        <v>706</v>
+        <v>704</v>
       </c>
       <c r="B374" s="1" t="s">
-        <v>779</v>
+        <v>777</v>
       </c>
       <c r="C374" s="4" t="s">
-        <v>780</v>
+        <v>778</v>
       </c>
       <c r="D374" s="5">
         <v>2.5</v>
@@ -10746,13 +10755,13 @@
     </row>
     <row r="375" spans="1:9">
       <c r="A375" s="1" t="s">
-        <v>706</v>
+        <v>704</v>
       </c>
       <c r="B375" s="1" t="s">
-        <v>781</v>
+        <v>779</v>
       </c>
       <c r="C375" s="4" t="s">
-        <v>782</v>
+        <v>780</v>
       </c>
       <c r="D375" s="5">
         <v>5</v>
@@ -10767,13 +10776,13 @@
     </row>
     <row r="376" spans="1:9">
       <c r="A376" s="1" t="s">
-        <v>706</v>
+        <v>704</v>
       </c>
       <c r="B376" s="1" t="s">
-        <v>783</v>
+        <v>781</v>
       </c>
       <c r="C376" s="4" t="s">
-        <v>784</v>
+        <v>782</v>
       </c>
       <c r="D376" s="5">
         <v>1</v>
@@ -10788,13 +10797,13 @@
     </row>
     <row r="377" spans="1:9">
       <c r="A377" s="1" t="s">
-        <v>706</v>
+        <v>704</v>
       </c>
       <c r="B377" s="1" t="s">
-        <v>785</v>
+        <v>783</v>
       </c>
       <c r="C377" s="4" t="s">
-        <v>786</v>
+        <v>784</v>
       </c>
       <c r="D377" s="5">
         <v>5</v>
@@ -10809,13 +10818,13 @@
     </row>
     <row r="378" spans="1:9">
       <c r="A378" s="1" t="s">
-        <v>706</v>
+        <v>704</v>
       </c>
       <c r="B378" s="1" t="s">
-        <v>787</v>
+        <v>785</v>
       </c>
       <c r="C378" s="4" t="s">
-        <v>788</v>
+        <v>786</v>
       </c>
       <c r="D378" s="5">
         <v>3</v>
@@ -10830,13 +10839,13 @@
     </row>
     <row r="379" spans="1:9">
       <c r="A379" s="1" t="s">
-        <v>706</v>
+        <v>704</v>
       </c>
       <c r="B379" s="1" t="s">
-        <v>789</v>
+        <v>787</v>
       </c>
       <c r="C379" s="4" t="s">
-        <v>790</v>
+        <v>788</v>
       </c>
       <c r="D379" s="5">
         <v>4</v>
@@ -10851,13 +10860,13 @@
     </row>
     <row r="380" spans="1:9">
       <c r="A380" s="1" t="s">
-        <v>706</v>
+        <v>704</v>
       </c>
       <c r="B380" s="1" t="s">
-        <v>791</v>
+        <v>789</v>
       </c>
       <c r="C380" s="4" t="s">
-        <v>792</v>
+        <v>790</v>
       </c>
       <c r="D380" s="5">
         <v>2.5</v>
@@ -10872,13 +10881,13 @@
     </row>
     <row r="381" spans="1:9">
       <c r="A381" s="1" t="s">
-        <v>706</v>
+        <v>704</v>
       </c>
       <c r="B381" s="1" t="s">
-        <v>793</v>
+        <v>791</v>
       </c>
       <c r="C381" s="4" t="s">
-        <v>794</v>
+        <v>792</v>
       </c>
       <c r="D381" s="5">
         <v>5</v>
@@ -10893,13 +10902,13 @@
     </row>
     <row r="382" spans="1:9">
       <c r="A382" s="1" t="s">
-        <v>706</v>
+        <v>704</v>
       </c>
       <c r="B382" s="1" t="s">
-        <v>795</v>
+        <v>793</v>
       </c>
       <c r="C382" s="4" t="s">
-        <v>796</v>
+        <v>794</v>
       </c>
       <c r="D382" s="5">
         <v>6.5</v>
@@ -10914,13 +10923,13 @@
     </row>
     <row r="383" spans="1:9">
       <c r="A383" s="1" t="s">
-        <v>706</v>
+        <v>704</v>
       </c>
       <c r="B383" s="1" t="s">
-        <v>797</v>
+        <v>795</v>
       </c>
       <c r="C383" s="4" t="s">
-        <v>798</v>
+        <v>796</v>
       </c>
       <c r="D383" s="5">
         <v>10</v>
@@ -10935,13 +10944,13 @@
     </row>
     <row r="384" spans="1:9">
       <c r="A384" s="1" t="s">
-        <v>706</v>
+        <v>704</v>
       </c>
       <c r="B384" s="1" t="s">
-        <v>799</v>
+        <v>797</v>
       </c>
       <c r="C384" s="4" t="s">
-        <v>800</v>
+        <v>798</v>
       </c>
       <c r="D384" s="5">
         <v>8</v>
@@ -10956,13 +10965,13 @@
     </row>
     <row r="385" spans="1:9">
       <c r="A385" s="1" t="s">
-        <v>706</v>
+        <v>704</v>
       </c>
       <c r="B385" s="1" t="s">
-        <v>801</v>
+        <v>799</v>
       </c>
       <c r="C385" s="4" t="s">
-        <v>802</v>
+        <v>800</v>
       </c>
       <c r="D385" s="5">
         <v>2</v>
@@ -10977,13 +10986,13 @@
     </row>
     <row r="386" spans="1:9">
       <c r="A386" s="1" t="s">
-        <v>706</v>
+        <v>704</v>
       </c>
       <c r="B386" s="1" t="s">
-        <v>803</v>
+        <v>801</v>
       </c>
       <c r="C386" s="4" t="s">
-        <v>804</v>
+        <v>802</v>
       </c>
       <c r="D386" s="5">
         <v>1</v>
@@ -10998,13 +11007,13 @@
     </row>
     <row r="387" spans="1:9">
       <c r="A387" s="1" t="s">
-        <v>706</v>
+        <v>704</v>
       </c>
       <c r="B387" s="1" t="s">
-        <v>805</v>
+        <v>803</v>
       </c>
       <c r="C387" s="4" t="s">
-        <v>806</v>
+        <v>804</v>
       </c>
       <c r="D387" s="5">
         <v>5</v>
@@ -11019,13 +11028,13 @@
     </row>
     <row r="388" spans="1:9">
       <c r="A388" s="1" t="s">
-        <v>706</v>
+        <v>704</v>
       </c>
       <c r="B388" s="1" t="s">
-        <v>807</v>
+        <v>805</v>
       </c>
       <c r="C388" s="4" t="s">
-        <v>808</v>
+        <v>806</v>
       </c>
       <c r="D388" s="5">
         <v>5</v>
@@ -11040,13 +11049,13 @@
     </row>
     <row r="389" spans="1:9">
       <c r="A389" s="1" t="s">
-        <v>706</v>
+        <v>704</v>
       </c>
       <c r="B389" s="1" t="s">
-        <v>809</v>
+        <v>807</v>
       </c>
       <c r="C389" s="4" t="s">
-        <v>810</v>
+        <v>808</v>
       </c>
       <c r="D389" s="5">
         <v>1</v>
@@ -11061,13 +11070,13 @@
     </row>
     <row r="390" spans="1:9">
       <c r="A390" s="1" t="s">
-        <v>706</v>
+        <v>704</v>
       </c>
       <c r="B390" s="1" t="s">
-        <v>811</v>
+        <v>809</v>
       </c>
       <c r="C390" s="4" t="s">
-        <v>812</v>
+        <v>810</v>
       </c>
       <c r="D390" s="5">
         <v>1</v>
@@ -11082,13 +11091,13 @@
     </row>
     <row r="391" spans="1:9">
       <c r="A391" s="1" t="s">
-        <v>706</v>
+        <v>704</v>
       </c>
       <c r="B391" s="1" t="s">
-        <v>813</v>
+        <v>811</v>
       </c>
       <c r="C391" s="4" t="s">
-        <v>814</v>
+        <v>812</v>
       </c>
       <c r="D391" s="5">
         <v>25</v>
@@ -11103,13 +11112,13 @@
     </row>
     <row r="392" spans="1:9">
       <c r="A392" s="1" t="s">
-        <v>706</v>
+        <v>704</v>
       </c>
       <c r="B392" s="1" t="s">
-        <v>815</v>
+        <v>813</v>
       </c>
       <c r="C392" s="4" t="s">
-        <v>816</v>
+        <v>814</v>
       </c>
       <c r="D392" s="5">
         <v>35</v>
@@ -11124,13 +11133,13 @@
     </row>
     <row r="393" spans="1:9">
       <c r="A393" s="1" t="s">
-        <v>706</v>
+        <v>704</v>
       </c>
       <c r="B393" s="1" t="s">
-        <v>817</v>
+        <v>815</v>
       </c>
       <c r="C393" s="4" t="s">
-        <v>818</v>
+        <v>816</v>
       </c>
       <c r="D393" s="5">
         <v>3</v>
@@ -11145,13 +11154,13 @@
     </row>
     <row r="394" spans="1:9">
       <c r="A394" s="1" t="s">
-        <v>706</v>
+        <v>704</v>
       </c>
       <c r="B394" s="1" t="s">
-        <v>819</v>
+        <v>817</v>
       </c>
       <c r="C394" s="4" t="s">
-        <v>820</v>
+        <v>818</v>
       </c>
       <c r="D394" s="5">
         <v>3</v>
@@ -11166,13 +11175,13 @@
     </row>
     <row r="395" spans="1:9">
       <c r="A395" s="1" t="s">
-        <v>706</v>
+        <v>704</v>
       </c>
       <c r="B395" s="1" t="s">
-        <v>821</v>
+        <v>819</v>
       </c>
       <c r="C395" s="4" t="s">
-        <v>822</v>
+        <v>820</v>
       </c>
       <c r="D395" s="5">
         <v>2</v>
@@ -11187,13 +11196,13 @@
     </row>
     <row r="396" spans="1:9">
       <c r="A396" s="1" t="s">
-        <v>706</v>
+        <v>704</v>
       </c>
       <c r="B396" s="1" t="s">
-        <v>823</v>
+        <v>821</v>
       </c>
       <c r="C396" s="4" t="s">
-        <v>824</v>
+        <v>822</v>
       </c>
       <c r="D396" s="5">
         <v>0.7</v>
@@ -11207,11 +11216,12 @@
       <c r="I396" s="1"/>
     </row>
   </sheetData>
+  <phoneticPr fontId="2" type="noConversion"/>
   <dataValidations count="2">
-    <dataValidation type="list" sqref="H2:H396" xr:uid="{00000000-0002-0000-0000-000000000000}">
+    <dataValidation type="list" sqref="H2:H141 H142:H396" xr:uid="{00000000-0002-0000-0000-000000000000}">
       <formula1>"taip,ne"</formula1>
     </dataValidation>
-    <dataValidation type="list" sqref="F2:F396" xr:uid="{00000000-0002-0000-0000-000001000000}">
+    <dataValidation type="list" sqref="F2:F141 F142:F396" xr:uid="{00000000-0002-0000-0000-000001000000}">
       <formula1>",dalinis,pilnas,brėžinys,fiksuotas"</formula1>
     </dataValidation>
   </dataValidations>
@@ -11233,10 +11243,10 @@
   <sheetData>
     <row r="1" spans="1:2" ht="15">
       <c r="A1" s="2" t="s">
-        <v>825</v>
+        <v>823</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>826</v>
+        <v>824</v>
       </c>
     </row>
     <row r="2" spans="1:2">
@@ -11244,7 +11254,7 @@
         <v>0</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>827</v>
+        <v>825</v>
       </c>
     </row>
     <row r="3" spans="1:2">
@@ -11252,7 +11262,7 @@
         <v>1</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>828</v>
+        <v>826</v>
       </c>
     </row>
     <row r="4" spans="1:2">
@@ -11260,7 +11270,7 @@
         <v>2</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>829</v>
+        <v>827</v>
       </c>
     </row>
     <row r="5" spans="1:2">
@@ -11268,7 +11278,7 @@
         <v>3</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>830</v>
+        <v>828</v>
       </c>
     </row>
     <row r="6" spans="1:2">
@@ -11276,7 +11286,7 @@
         <v>4</v>
       </c>
       <c r="B6" s="1" t="s">
-        <v>831</v>
+        <v>829</v>
       </c>
     </row>
     <row r="7" spans="1:2">
@@ -11284,7 +11294,7 @@
         <v>5</v>
       </c>
       <c r="B7" s="1" t="s">
-        <v>832</v>
+        <v>830</v>
       </c>
     </row>
     <row r="8" spans="1:2">
@@ -11292,7 +11302,7 @@
         <v>6</v>
       </c>
       <c r="B8" s="1" t="s">
-        <v>833</v>
+        <v>831</v>
       </c>
     </row>
     <row r="9" spans="1:2">
@@ -11300,7 +11310,7 @@
         <v>7</v>
       </c>
       <c r="B9" s="1" t="s">
-        <v>834</v>
+        <v>832</v>
       </c>
     </row>
     <row r="10" spans="1:2">
@@ -11308,15 +11318,15 @@
         <v>8</v>
       </c>
       <c r="B10" s="1" t="s">
-        <v>835</v>
+        <v>833</v>
       </c>
     </row>
     <row r="11" spans="1:2">
       <c r="A11" s="1" t="s">
-        <v>836</v>
+        <v>834</v>
       </c>
       <c r="B11" s="1" t="s">
-        <v>837</v>
+        <v>835</v>
       </c>
     </row>
     <row r="12" spans="1:2">

</xml_diff>

<commit_message>
Update wide format order, bleed options and layout performance
</commit_message>
<xml_diff>
--- a/data/copypro_kodai.xlsx
+++ b/data/copypro_kodai.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\deima\Downloads\copypro_tools_final_github_bundle\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{62E82CA7-65C5-4A0D-B296-E24DAC4FE08E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{82D11921-BB20-4B9B-8848-F86994760BC9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -5871,7 +5871,7 @@
         <v>303</v>
       </c>
       <c r="D142" s="5">
-        <v>1.8</v>
+        <v>3.6</v>
       </c>
       <c r="E142" s="1"/>
       <c r="F142" s="1" t="s">

</xml_diff>